<commit_message>
new changes in Pool
</commit_message>
<xml_diff>
--- a/ranking/results.xlsx
+++ b/ranking/results.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BI8"/>
+  <dimension ref="A1:JC10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -734,6 +734,1016 @@
           <t>theta_9_dgd</t>
         </is>
       </c>
+      <c r="BJ1" s="1" t="inlineStr">
+        <is>
+          <t>F1_Proposed</t>
+        </is>
+      </c>
+      <c r="BK1" s="1" t="inlineStr">
+        <is>
+          <t>Kendall_Proposed</t>
+        </is>
+      </c>
+      <c r="BL1" s="1" t="inlineStr">
+        <is>
+          <t>theta_10_true</t>
+        </is>
+      </c>
+      <c r="BM1" s="1" t="inlineStr">
+        <is>
+          <t>theta_10_uadmm</t>
+        </is>
+      </c>
+      <c r="BN1" s="1" t="inlineStr">
+        <is>
+          <t>theta_10_local</t>
+        </is>
+      </c>
+      <c r="BO1" s="1" t="inlineStr">
+        <is>
+          <t>theta_10_pooled</t>
+        </is>
+      </c>
+      <c r="BP1" s="1" t="inlineStr">
+        <is>
+          <t>theta_10_dgd</t>
+        </is>
+      </c>
+      <c r="BQ1" s="1" t="inlineStr">
+        <is>
+          <t>theta_11_true</t>
+        </is>
+      </c>
+      <c r="BR1" s="1" t="inlineStr">
+        <is>
+          <t>theta_11_uadmm</t>
+        </is>
+      </c>
+      <c r="BS1" s="1" t="inlineStr">
+        <is>
+          <t>theta_11_local</t>
+        </is>
+      </c>
+      <c r="BT1" s="1" t="inlineStr">
+        <is>
+          <t>theta_11_pooled</t>
+        </is>
+      </c>
+      <c r="BU1" s="1" t="inlineStr">
+        <is>
+          <t>theta_11_dgd</t>
+        </is>
+      </c>
+      <c r="BV1" s="1" t="inlineStr">
+        <is>
+          <t>theta_12_true</t>
+        </is>
+      </c>
+      <c r="BW1" s="1" t="inlineStr">
+        <is>
+          <t>theta_12_uadmm</t>
+        </is>
+      </c>
+      <c r="BX1" s="1" t="inlineStr">
+        <is>
+          <t>theta_12_local</t>
+        </is>
+      </c>
+      <c r="BY1" s="1" t="inlineStr">
+        <is>
+          <t>theta_12_pooled</t>
+        </is>
+      </c>
+      <c r="BZ1" s="1" t="inlineStr">
+        <is>
+          <t>theta_12_dgd</t>
+        </is>
+      </c>
+      <c r="CA1" s="1" t="inlineStr">
+        <is>
+          <t>theta_13_true</t>
+        </is>
+      </c>
+      <c r="CB1" s="1" t="inlineStr">
+        <is>
+          <t>theta_13_uadmm</t>
+        </is>
+      </c>
+      <c r="CC1" s="1" t="inlineStr">
+        <is>
+          <t>theta_13_local</t>
+        </is>
+      </c>
+      <c r="CD1" s="1" t="inlineStr">
+        <is>
+          <t>theta_13_pooled</t>
+        </is>
+      </c>
+      <c r="CE1" s="1" t="inlineStr">
+        <is>
+          <t>theta_13_dgd</t>
+        </is>
+      </c>
+      <c r="CF1" s="1" t="inlineStr">
+        <is>
+          <t>theta_14_true</t>
+        </is>
+      </c>
+      <c r="CG1" s="1" t="inlineStr">
+        <is>
+          <t>theta_14_uadmm</t>
+        </is>
+      </c>
+      <c r="CH1" s="1" t="inlineStr">
+        <is>
+          <t>theta_14_local</t>
+        </is>
+      </c>
+      <c r="CI1" s="1" t="inlineStr">
+        <is>
+          <t>theta_14_pooled</t>
+        </is>
+      </c>
+      <c r="CJ1" s="1" t="inlineStr">
+        <is>
+          <t>theta_14_dgd</t>
+        </is>
+      </c>
+      <c r="CK1" s="1" t="inlineStr">
+        <is>
+          <t>theta_15_true</t>
+        </is>
+      </c>
+      <c r="CL1" s="1" t="inlineStr">
+        <is>
+          <t>theta_15_uadmm</t>
+        </is>
+      </c>
+      <c r="CM1" s="1" t="inlineStr">
+        <is>
+          <t>theta_15_local</t>
+        </is>
+      </c>
+      <c r="CN1" s="1" t="inlineStr">
+        <is>
+          <t>theta_15_pooled</t>
+        </is>
+      </c>
+      <c r="CO1" s="1" t="inlineStr">
+        <is>
+          <t>theta_15_dgd</t>
+        </is>
+      </c>
+      <c r="CP1" s="1" t="inlineStr">
+        <is>
+          <t>theta_16_true</t>
+        </is>
+      </c>
+      <c r="CQ1" s="1" t="inlineStr">
+        <is>
+          <t>theta_16_uadmm</t>
+        </is>
+      </c>
+      <c r="CR1" s="1" t="inlineStr">
+        <is>
+          <t>theta_16_local</t>
+        </is>
+      </c>
+      <c r="CS1" s="1" t="inlineStr">
+        <is>
+          <t>theta_16_pooled</t>
+        </is>
+      </c>
+      <c r="CT1" s="1" t="inlineStr">
+        <is>
+          <t>theta_16_dgd</t>
+        </is>
+      </c>
+      <c r="CU1" s="1" t="inlineStr">
+        <is>
+          <t>theta_17_true</t>
+        </is>
+      </c>
+      <c r="CV1" s="1" t="inlineStr">
+        <is>
+          <t>theta_17_uadmm</t>
+        </is>
+      </c>
+      <c r="CW1" s="1" t="inlineStr">
+        <is>
+          <t>theta_17_local</t>
+        </is>
+      </c>
+      <c r="CX1" s="1" t="inlineStr">
+        <is>
+          <t>theta_17_pooled</t>
+        </is>
+      </c>
+      <c r="CY1" s="1" t="inlineStr">
+        <is>
+          <t>theta_17_dgd</t>
+        </is>
+      </c>
+      <c r="CZ1" s="1" t="inlineStr">
+        <is>
+          <t>theta_18_true</t>
+        </is>
+      </c>
+      <c r="DA1" s="1" t="inlineStr">
+        <is>
+          <t>theta_18_uadmm</t>
+        </is>
+      </c>
+      <c r="DB1" s="1" t="inlineStr">
+        <is>
+          <t>theta_18_local</t>
+        </is>
+      </c>
+      <c r="DC1" s="1" t="inlineStr">
+        <is>
+          <t>theta_18_pooled</t>
+        </is>
+      </c>
+      <c r="DD1" s="1" t="inlineStr">
+        <is>
+          <t>theta_18_dgd</t>
+        </is>
+      </c>
+      <c r="DE1" s="1" t="inlineStr">
+        <is>
+          <t>theta_19_true</t>
+        </is>
+      </c>
+      <c r="DF1" s="1" t="inlineStr">
+        <is>
+          <t>theta_19_uadmm</t>
+        </is>
+      </c>
+      <c r="DG1" s="1" t="inlineStr">
+        <is>
+          <t>theta_19_local</t>
+        </is>
+      </c>
+      <c r="DH1" s="1" t="inlineStr">
+        <is>
+          <t>theta_19_pooled</t>
+        </is>
+      </c>
+      <c r="DI1" s="1" t="inlineStr">
+        <is>
+          <t>theta_19_dgd</t>
+        </is>
+      </c>
+      <c r="DJ1" s="1" t="inlineStr">
+        <is>
+          <t>theta_20_true</t>
+        </is>
+      </c>
+      <c r="DK1" s="1" t="inlineStr">
+        <is>
+          <t>theta_20_uadmm</t>
+        </is>
+      </c>
+      <c r="DL1" s="1" t="inlineStr">
+        <is>
+          <t>theta_20_local</t>
+        </is>
+      </c>
+      <c r="DM1" s="1" t="inlineStr">
+        <is>
+          <t>theta_20_pooled</t>
+        </is>
+      </c>
+      <c r="DN1" s="1" t="inlineStr">
+        <is>
+          <t>theta_20_dgd</t>
+        </is>
+      </c>
+      <c r="DO1" s="1" t="inlineStr">
+        <is>
+          <t>theta_21_true</t>
+        </is>
+      </c>
+      <c r="DP1" s="1" t="inlineStr">
+        <is>
+          <t>theta_21_uadmm</t>
+        </is>
+      </c>
+      <c r="DQ1" s="1" t="inlineStr">
+        <is>
+          <t>theta_21_local</t>
+        </is>
+      </c>
+      <c r="DR1" s="1" t="inlineStr">
+        <is>
+          <t>theta_21_pooled</t>
+        </is>
+      </c>
+      <c r="DS1" s="1" t="inlineStr">
+        <is>
+          <t>theta_21_dgd</t>
+        </is>
+      </c>
+      <c r="DT1" s="1" t="inlineStr">
+        <is>
+          <t>theta_22_true</t>
+        </is>
+      </c>
+      <c r="DU1" s="1" t="inlineStr">
+        <is>
+          <t>theta_22_uadmm</t>
+        </is>
+      </c>
+      <c r="DV1" s="1" t="inlineStr">
+        <is>
+          <t>theta_22_local</t>
+        </is>
+      </c>
+      <c r="DW1" s="1" t="inlineStr">
+        <is>
+          <t>theta_22_pooled</t>
+        </is>
+      </c>
+      <c r="DX1" s="1" t="inlineStr">
+        <is>
+          <t>theta_22_dgd</t>
+        </is>
+      </c>
+      <c r="DY1" s="1" t="inlineStr">
+        <is>
+          <t>theta_23_true</t>
+        </is>
+      </c>
+      <c r="DZ1" s="1" t="inlineStr">
+        <is>
+          <t>theta_23_uadmm</t>
+        </is>
+      </c>
+      <c r="EA1" s="1" t="inlineStr">
+        <is>
+          <t>theta_23_local</t>
+        </is>
+      </c>
+      <c r="EB1" s="1" t="inlineStr">
+        <is>
+          <t>theta_23_pooled</t>
+        </is>
+      </c>
+      <c r="EC1" s="1" t="inlineStr">
+        <is>
+          <t>theta_23_dgd</t>
+        </is>
+      </c>
+      <c r="ED1" s="1" t="inlineStr">
+        <is>
+          <t>theta_24_true</t>
+        </is>
+      </c>
+      <c r="EE1" s="1" t="inlineStr">
+        <is>
+          <t>theta_24_uadmm</t>
+        </is>
+      </c>
+      <c r="EF1" s="1" t="inlineStr">
+        <is>
+          <t>theta_24_local</t>
+        </is>
+      </c>
+      <c r="EG1" s="1" t="inlineStr">
+        <is>
+          <t>theta_24_pooled</t>
+        </is>
+      </c>
+      <c r="EH1" s="1" t="inlineStr">
+        <is>
+          <t>theta_24_dgd</t>
+        </is>
+      </c>
+      <c r="EI1" s="1" t="inlineStr">
+        <is>
+          <t>theta_25_true</t>
+        </is>
+      </c>
+      <c r="EJ1" s="1" t="inlineStr">
+        <is>
+          <t>theta_25_uadmm</t>
+        </is>
+      </c>
+      <c r="EK1" s="1" t="inlineStr">
+        <is>
+          <t>theta_25_local</t>
+        </is>
+      </c>
+      <c r="EL1" s="1" t="inlineStr">
+        <is>
+          <t>theta_25_pooled</t>
+        </is>
+      </c>
+      <c r="EM1" s="1" t="inlineStr">
+        <is>
+          <t>theta_25_dgd</t>
+        </is>
+      </c>
+      <c r="EN1" s="1" t="inlineStr">
+        <is>
+          <t>theta_26_true</t>
+        </is>
+      </c>
+      <c r="EO1" s="1" t="inlineStr">
+        <is>
+          <t>theta_26_uadmm</t>
+        </is>
+      </c>
+      <c r="EP1" s="1" t="inlineStr">
+        <is>
+          <t>theta_26_local</t>
+        </is>
+      </c>
+      <c r="EQ1" s="1" t="inlineStr">
+        <is>
+          <t>theta_26_pooled</t>
+        </is>
+      </c>
+      <c r="ER1" s="1" t="inlineStr">
+        <is>
+          <t>theta_26_dgd</t>
+        </is>
+      </c>
+      <c r="ES1" s="1" t="inlineStr">
+        <is>
+          <t>theta_27_true</t>
+        </is>
+      </c>
+      <c r="ET1" s="1" t="inlineStr">
+        <is>
+          <t>theta_27_uadmm</t>
+        </is>
+      </c>
+      <c r="EU1" s="1" t="inlineStr">
+        <is>
+          <t>theta_27_local</t>
+        </is>
+      </c>
+      <c r="EV1" s="1" t="inlineStr">
+        <is>
+          <t>theta_27_pooled</t>
+        </is>
+      </c>
+      <c r="EW1" s="1" t="inlineStr">
+        <is>
+          <t>theta_27_dgd</t>
+        </is>
+      </c>
+      <c r="EX1" s="1" t="inlineStr">
+        <is>
+          <t>theta_28_true</t>
+        </is>
+      </c>
+      <c r="EY1" s="1" t="inlineStr">
+        <is>
+          <t>theta_28_uadmm</t>
+        </is>
+      </c>
+      <c r="EZ1" s="1" t="inlineStr">
+        <is>
+          <t>theta_28_local</t>
+        </is>
+      </c>
+      <c r="FA1" s="1" t="inlineStr">
+        <is>
+          <t>theta_28_pooled</t>
+        </is>
+      </c>
+      <c r="FB1" s="1" t="inlineStr">
+        <is>
+          <t>theta_28_dgd</t>
+        </is>
+      </c>
+      <c r="FC1" s="1" t="inlineStr">
+        <is>
+          <t>theta_29_true</t>
+        </is>
+      </c>
+      <c r="FD1" s="1" t="inlineStr">
+        <is>
+          <t>theta_29_uadmm</t>
+        </is>
+      </c>
+      <c r="FE1" s="1" t="inlineStr">
+        <is>
+          <t>theta_29_local</t>
+        </is>
+      </c>
+      <c r="FF1" s="1" t="inlineStr">
+        <is>
+          <t>theta_29_pooled</t>
+        </is>
+      </c>
+      <c r="FG1" s="1" t="inlineStr">
+        <is>
+          <t>theta_29_dgd</t>
+        </is>
+      </c>
+      <c r="FH1" s="1" t="inlineStr">
+        <is>
+          <t>theta_30_true</t>
+        </is>
+      </c>
+      <c r="FI1" s="1" t="inlineStr">
+        <is>
+          <t>theta_30_uadmm</t>
+        </is>
+      </c>
+      <c r="FJ1" s="1" t="inlineStr">
+        <is>
+          <t>theta_30_local</t>
+        </is>
+      </c>
+      <c r="FK1" s="1" t="inlineStr">
+        <is>
+          <t>theta_30_pooled</t>
+        </is>
+      </c>
+      <c r="FL1" s="1" t="inlineStr">
+        <is>
+          <t>theta_30_dgd</t>
+        </is>
+      </c>
+      <c r="FM1" s="1" t="inlineStr">
+        <is>
+          <t>theta_31_true</t>
+        </is>
+      </c>
+      <c r="FN1" s="1" t="inlineStr">
+        <is>
+          <t>theta_31_uadmm</t>
+        </is>
+      </c>
+      <c r="FO1" s="1" t="inlineStr">
+        <is>
+          <t>theta_31_local</t>
+        </is>
+      </c>
+      <c r="FP1" s="1" t="inlineStr">
+        <is>
+          <t>theta_31_pooled</t>
+        </is>
+      </c>
+      <c r="FQ1" s="1" t="inlineStr">
+        <is>
+          <t>theta_31_dgd</t>
+        </is>
+      </c>
+      <c r="FR1" s="1" t="inlineStr">
+        <is>
+          <t>theta_32_true</t>
+        </is>
+      </c>
+      <c r="FS1" s="1" t="inlineStr">
+        <is>
+          <t>theta_32_uadmm</t>
+        </is>
+      </c>
+      <c r="FT1" s="1" t="inlineStr">
+        <is>
+          <t>theta_32_local</t>
+        </is>
+      </c>
+      <c r="FU1" s="1" t="inlineStr">
+        <is>
+          <t>theta_32_pooled</t>
+        </is>
+      </c>
+      <c r="FV1" s="1" t="inlineStr">
+        <is>
+          <t>theta_32_dgd</t>
+        </is>
+      </c>
+      <c r="FW1" s="1" t="inlineStr">
+        <is>
+          <t>theta_33_true</t>
+        </is>
+      </c>
+      <c r="FX1" s="1" t="inlineStr">
+        <is>
+          <t>theta_33_uadmm</t>
+        </is>
+      </c>
+      <c r="FY1" s="1" t="inlineStr">
+        <is>
+          <t>theta_33_local</t>
+        </is>
+      </c>
+      <c r="FZ1" s="1" t="inlineStr">
+        <is>
+          <t>theta_33_pooled</t>
+        </is>
+      </c>
+      <c r="GA1" s="1" t="inlineStr">
+        <is>
+          <t>theta_33_dgd</t>
+        </is>
+      </c>
+      <c r="GB1" s="1" t="inlineStr">
+        <is>
+          <t>theta_34_true</t>
+        </is>
+      </c>
+      <c r="GC1" s="1" t="inlineStr">
+        <is>
+          <t>theta_34_uadmm</t>
+        </is>
+      </c>
+      <c r="GD1" s="1" t="inlineStr">
+        <is>
+          <t>theta_34_local</t>
+        </is>
+      </c>
+      <c r="GE1" s="1" t="inlineStr">
+        <is>
+          <t>theta_34_pooled</t>
+        </is>
+      </c>
+      <c r="GF1" s="1" t="inlineStr">
+        <is>
+          <t>theta_34_dgd</t>
+        </is>
+      </c>
+      <c r="GG1" s="1" t="inlineStr">
+        <is>
+          <t>theta_35_true</t>
+        </is>
+      </c>
+      <c r="GH1" s="1" t="inlineStr">
+        <is>
+          <t>theta_35_uadmm</t>
+        </is>
+      </c>
+      <c r="GI1" s="1" t="inlineStr">
+        <is>
+          <t>theta_35_local</t>
+        </is>
+      </c>
+      <c r="GJ1" s="1" t="inlineStr">
+        <is>
+          <t>theta_35_pooled</t>
+        </is>
+      </c>
+      <c r="GK1" s="1" t="inlineStr">
+        <is>
+          <t>theta_35_dgd</t>
+        </is>
+      </c>
+      <c r="GL1" s="1" t="inlineStr">
+        <is>
+          <t>theta_36_true</t>
+        </is>
+      </c>
+      <c r="GM1" s="1" t="inlineStr">
+        <is>
+          <t>theta_36_uadmm</t>
+        </is>
+      </c>
+      <c r="GN1" s="1" t="inlineStr">
+        <is>
+          <t>theta_36_local</t>
+        </is>
+      </c>
+      <c r="GO1" s="1" t="inlineStr">
+        <is>
+          <t>theta_36_pooled</t>
+        </is>
+      </c>
+      <c r="GP1" s="1" t="inlineStr">
+        <is>
+          <t>theta_36_dgd</t>
+        </is>
+      </c>
+      <c r="GQ1" s="1" t="inlineStr">
+        <is>
+          <t>theta_37_true</t>
+        </is>
+      </c>
+      <c r="GR1" s="1" t="inlineStr">
+        <is>
+          <t>theta_37_uadmm</t>
+        </is>
+      </c>
+      <c r="GS1" s="1" t="inlineStr">
+        <is>
+          <t>theta_37_local</t>
+        </is>
+      </c>
+      <c r="GT1" s="1" t="inlineStr">
+        <is>
+          <t>theta_37_pooled</t>
+        </is>
+      </c>
+      <c r="GU1" s="1" t="inlineStr">
+        <is>
+          <t>theta_37_dgd</t>
+        </is>
+      </c>
+      <c r="GV1" s="1" t="inlineStr">
+        <is>
+          <t>theta_38_true</t>
+        </is>
+      </c>
+      <c r="GW1" s="1" t="inlineStr">
+        <is>
+          <t>theta_38_uadmm</t>
+        </is>
+      </c>
+      <c r="GX1" s="1" t="inlineStr">
+        <is>
+          <t>theta_38_local</t>
+        </is>
+      </c>
+      <c r="GY1" s="1" t="inlineStr">
+        <is>
+          <t>theta_38_pooled</t>
+        </is>
+      </c>
+      <c r="GZ1" s="1" t="inlineStr">
+        <is>
+          <t>theta_38_dgd</t>
+        </is>
+      </c>
+      <c r="HA1" s="1" t="inlineStr">
+        <is>
+          <t>theta_39_true</t>
+        </is>
+      </c>
+      <c r="HB1" s="1" t="inlineStr">
+        <is>
+          <t>theta_39_uadmm</t>
+        </is>
+      </c>
+      <c r="HC1" s="1" t="inlineStr">
+        <is>
+          <t>theta_39_local</t>
+        </is>
+      </c>
+      <c r="HD1" s="1" t="inlineStr">
+        <is>
+          <t>theta_39_pooled</t>
+        </is>
+      </c>
+      <c r="HE1" s="1" t="inlineStr">
+        <is>
+          <t>theta_39_dgd</t>
+        </is>
+      </c>
+      <c r="HF1" s="1" t="inlineStr">
+        <is>
+          <t>theta_40_true</t>
+        </is>
+      </c>
+      <c r="HG1" s="1" t="inlineStr">
+        <is>
+          <t>theta_40_uadmm</t>
+        </is>
+      </c>
+      <c r="HH1" s="1" t="inlineStr">
+        <is>
+          <t>theta_40_local</t>
+        </is>
+      </c>
+      <c r="HI1" s="1" t="inlineStr">
+        <is>
+          <t>theta_40_pooled</t>
+        </is>
+      </c>
+      <c r="HJ1" s="1" t="inlineStr">
+        <is>
+          <t>theta_40_dgd</t>
+        </is>
+      </c>
+      <c r="HK1" s="1" t="inlineStr">
+        <is>
+          <t>theta_41_true</t>
+        </is>
+      </c>
+      <c r="HL1" s="1" t="inlineStr">
+        <is>
+          <t>theta_41_uadmm</t>
+        </is>
+      </c>
+      <c r="HM1" s="1" t="inlineStr">
+        <is>
+          <t>theta_41_local</t>
+        </is>
+      </c>
+      <c r="HN1" s="1" t="inlineStr">
+        <is>
+          <t>theta_41_pooled</t>
+        </is>
+      </c>
+      <c r="HO1" s="1" t="inlineStr">
+        <is>
+          <t>theta_41_dgd</t>
+        </is>
+      </c>
+      <c r="HP1" s="1" t="inlineStr">
+        <is>
+          <t>theta_42_true</t>
+        </is>
+      </c>
+      <c r="HQ1" s="1" t="inlineStr">
+        <is>
+          <t>theta_42_uadmm</t>
+        </is>
+      </c>
+      <c r="HR1" s="1" t="inlineStr">
+        <is>
+          <t>theta_42_local</t>
+        </is>
+      </c>
+      <c r="HS1" s="1" t="inlineStr">
+        <is>
+          <t>theta_42_pooled</t>
+        </is>
+      </c>
+      <c r="HT1" s="1" t="inlineStr">
+        <is>
+          <t>theta_42_dgd</t>
+        </is>
+      </c>
+      <c r="HU1" s="1" t="inlineStr">
+        <is>
+          <t>theta_43_true</t>
+        </is>
+      </c>
+      <c r="HV1" s="1" t="inlineStr">
+        <is>
+          <t>theta_43_uadmm</t>
+        </is>
+      </c>
+      <c r="HW1" s="1" t="inlineStr">
+        <is>
+          <t>theta_43_local</t>
+        </is>
+      </c>
+      <c r="HX1" s="1" t="inlineStr">
+        <is>
+          <t>theta_43_pooled</t>
+        </is>
+      </c>
+      <c r="HY1" s="1" t="inlineStr">
+        <is>
+          <t>theta_43_dgd</t>
+        </is>
+      </c>
+      <c r="HZ1" s="1" t="inlineStr">
+        <is>
+          <t>theta_44_true</t>
+        </is>
+      </c>
+      <c r="IA1" s="1" t="inlineStr">
+        <is>
+          <t>theta_44_uadmm</t>
+        </is>
+      </c>
+      <c r="IB1" s="1" t="inlineStr">
+        <is>
+          <t>theta_44_local</t>
+        </is>
+      </c>
+      <c r="IC1" s="1" t="inlineStr">
+        <is>
+          <t>theta_44_pooled</t>
+        </is>
+      </c>
+      <c r="ID1" s="1" t="inlineStr">
+        <is>
+          <t>theta_44_dgd</t>
+        </is>
+      </c>
+      <c r="IE1" s="1" t="inlineStr">
+        <is>
+          <t>theta_45_true</t>
+        </is>
+      </c>
+      <c r="IF1" s="1" t="inlineStr">
+        <is>
+          <t>theta_45_uadmm</t>
+        </is>
+      </c>
+      <c r="IG1" s="1" t="inlineStr">
+        <is>
+          <t>theta_45_local</t>
+        </is>
+      </c>
+      <c r="IH1" s="1" t="inlineStr">
+        <is>
+          <t>theta_45_pooled</t>
+        </is>
+      </c>
+      <c r="II1" s="1" t="inlineStr">
+        <is>
+          <t>theta_45_dgd</t>
+        </is>
+      </c>
+      <c r="IJ1" s="1" t="inlineStr">
+        <is>
+          <t>theta_46_true</t>
+        </is>
+      </c>
+      <c r="IK1" s="1" t="inlineStr">
+        <is>
+          <t>theta_46_uadmm</t>
+        </is>
+      </c>
+      <c r="IL1" s="1" t="inlineStr">
+        <is>
+          <t>theta_46_local</t>
+        </is>
+      </c>
+      <c r="IM1" s="1" t="inlineStr">
+        <is>
+          <t>theta_46_pooled</t>
+        </is>
+      </c>
+      <c r="IN1" s="1" t="inlineStr">
+        <is>
+          <t>theta_46_dgd</t>
+        </is>
+      </c>
+      <c r="IO1" s="1" t="inlineStr">
+        <is>
+          <t>theta_47_true</t>
+        </is>
+      </c>
+      <c r="IP1" s="1" t="inlineStr">
+        <is>
+          <t>theta_47_uadmm</t>
+        </is>
+      </c>
+      <c r="IQ1" s="1" t="inlineStr">
+        <is>
+          <t>theta_47_local</t>
+        </is>
+      </c>
+      <c r="IR1" s="1" t="inlineStr">
+        <is>
+          <t>theta_47_pooled</t>
+        </is>
+      </c>
+      <c r="IS1" s="1" t="inlineStr">
+        <is>
+          <t>theta_47_dgd</t>
+        </is>
+      </c>
+      <c r="IT1" s="1" t="inlineStr">
+        <is>
+          <t>theta_48_true</t>
+        </is>
+      </c>
+      <c r="IU1" s="1" t="inlineStr">
+        <is>
+          <t>theta_48_uadmm</t>
+        </is>
+      </c>
+      <c r="IV1" s="1" t="inlineStr">
+        <is>
+          <t>theta_48_local</t>
+        </is>
+      </c>
+      <c r="IW1" s="1" t="inlineStr">
+        <is>
+          <t>theta_48_pooled</t>
+        </is>
+      </c>
+      <c r="IX1" s="1" t="inlineStr">
+        <is>
+          <t>theta_48_dgd</t>
+        </is>
+      </c>
+      <c r="IY1" s="1" t="inlineStr">
+        <is>
+          <t>theta_49_true</t>
+        </is>
+      </c>
+      <c r="IZ1" s="1" t="inlineStr">
+        <is>
+          <t>theta_49_uadmm</t>
+        </is>
+      </c>
+      <c r="JA1" s="1" t="inlineStr">
+        <is>
+          <t>theta_49_local</t>
+        </is>
+      </c>
+      <c r="JB1" s="1" t="inlineStr">
+        <is>
+          <t>theta_49_pooled</t>
+        </is>
+      </c>
+      <c r="JC1" s="1" t="inlineStr">
+        <is>
+          <t>theta_49_dgd</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -923,6 +1933,208 @@
       <c r="BI2" t="n">
         <v>0.1212439507557961</v>
       </c>
+      <c r="BJ2" t="inlineStr"/>
+      <c r="BK2" t="inlineStr"/>
+      <c r="BL2" t="inlineStr"/>
+      <c r="BM2" t="inlineStr"/>
+      <c r="BN2" t="inlineStr"/>
+      <c r="BO2" t="inlineStr"/>
+      <c r="BP2" t="inlineStr"/>
+      <c r="BQ2" t="inlineStr"/>
+      <c r="BR2" t="inlineStr"/>
+      <c r="BS2" t="inlineStr"/>
+      <c r="BT2" t="inlineStr"/>
+      <c r="BU2" t="inlineStr"/>
+      <c r="BV2" t="inlineStr"/>
+      <c r="BW2" t="inlineStr"/>
+      <c r="BX2" t="inlineStr"/>
+      <c r="BY2" t="inlineStr"/>
+      <c r="BZ2" t="inlineStr"/>
+      <c r="CA2" t="inlineStr"/>
+      <c r="CB2" t="inlineStr"/>
+      <c r="CC2" t="inlineStr"/>
+      <c r="CD2" t="inlineStr"/>
+      <c r="CE2" t="inlineStr"/>
+      <c r="CF2" t="inlineStr"/>
+      <c r="CG2" t="inlineStr"/>
+      <c r="CH2" t="inlineStr"/>
+      <c r="CI2" t="inlineStr"/>
+      <c r="CJ2" t="inlineStr"/>
+      <c r="CK2" t="inlineStr"/>
+      <c r="CL2" t="inlineStr"/>
+      <c r="CM2" t="inlineStr"/>
+      <c r="CN2" t="inlineStr"/>
+      <c r="CO2" t="inlineStr"/>
+      <c r="CP2" t="inlineStr"/>
+      <c r="CQ2" t="inlineStr"/>
+      <c r="CR2" t="inlineStr"/>
+      <c r="CS2" t="inlineStr"/>
+      <c r="CT2" t="inlineStr"/>
+      <c r="CU2" t="inlineStr"/>
+      <c r="CV2" t="inlineStr"/>
+      <c r="CW2" t="inlineStr"/>
+      <c r="CX2" t="inlineStr"/>
+      <c r="CY2" t="inlineStr"/>
+      <c r="CZ2" t="inlineStr"/>
+      <c r="DA2" t="inlineStr"/>
+      <c r="DB2" t="inlineStr"/>
+      <c r="DC2" t="inlineStr"/>
+      <c r="DD2" t="inlineStr"/>
+      <c r="DE2" t="inlineStr"/>
+      <c r="DF2" t="inlineStr"/>
+      <c r="DG2" t="inlineStr"/>
+      <c r="DH2" t="inlineStr"/>
+      <c r="DI2" t="inlineStr"/>
+      <c r="DJ2" t="inlineStr"/>
+      <c r="DK2" t="inlineStr"/>
+      <c r="DL2" t="inlineStr"/>
+      <c r="DM2" t="inlineStr"/>
+      <c r="DN2" t="inlineStr"/>
+      <c r="DO2" t="inlineStr"/>
+      <c r="DP2" t="inlineStr"/>
+      <c r="DQ2" t="inlineStr"/>
+      <c r="DR2" t="inlineStr"/>
+      <c r="DS2" t="inlineStr"/>
+      <c r="DT2" t="inlineStr"/>
+      <c r="DU2" t="inlineStr"/>
+      <c r="DV2" t="inlineStr"/>
+      <c r="DW2" t="inlineStr"/>
+      <c r="DX2" t="inlineStr"/>
+      <c r="DY2" t="inlineStr"/>
+      <c r="DZ2" t="inlineStr"/>
+      <c r="EA2" t="inlineStr"/>
+      <c r="EB2" t="inlineStr"/>
+      <c r="EC2" t="inlineStr"/>
+      <c r="ED2" t="inlineStr"/>
+      <c r="EE2" t="inlineStr"/>
+      <c r="EF2" t="inlineStr"/>
+      <c r="EG2" t="inlineStr"/>
+      <c r="EH2" t="inlineStr"/>
+      <c r="EI2" t="inlineStr"/>
+      <c r="EJ2" t="inlineStr"/>
+      <c r="EK2" t="inlineStr"/>
+      <c r="EL2" t="inlineStr"/>
+      <c r="EM2" t="inlineStr"/>
+      <c r="EN2" t="inlineStr"/>
+      <c r="EO2" t="inlineStr"/>
+      <c r="EP2" t="inlineStr"/>
+      <c r="EQ2" t="inlineStr"/>
+      <c r="ER2" t="inlineStr"/>
+      <c r="ES2" t="inlineStr"/>
+      <c r="ET2" t="inlineStr"/>
+      <c r="EU2" t="inlineStr"/>
+      <c r="EV2" t="inlineStr"/>
+      <c r="EW2" t="inlineStr"/>
+      <c r="EX2" t="inlineStr"/>
+      <c r="EY2" t="inlineStr"/>
+      <c r="EZ2" t="inlineStr"/>
+      <c r="FA2" t="inlineStr"/>
+      <c r="FB2" t="inlineStr"/>
+      <c r="FC2" t="inlineStr"/>
+      <c r="FD2" t="inlineStr"/>
+      <c r="FE2" t="inlineStr"/>
+      <c r="FF2" t="inlineStr"/>
+      <c r="FG2" t="inlineStr"/>
+      <c r="FH2" t="inlineStr"/>
+      <c r="FI2" t="inlineStr"/>
+      <c r="FJ2" t="inlineStr"/>
+      <c r="FK2" t="inlineStr"/>
+      <c r="FL2" t="inlineStr"/>
+      <c r="FM2" t="inlineStr"/>
+      <c r="FN2" t="inlineStr"/>
+      <c r="FO2" t="inlineStr"/>
+      <c r="FP2" t="inlineStr"/>
+      <c r="FQ2" t="inlineStr"/>
+      <c r="FR2" t="inlineStr"/>
+      <c r="FS2" t="inlineStr"/>
+      <c r="FT2" t="inlineStr"/>
+      <c r="FU2" t="inlineStr"/>
+      <c r="FV2" t="inlineStr"/>
+      <c r="FW2" t="inlineStr"/>
+      <c r="FX2" t="inlineStr"/>
+      <c r="FY2" t="inlineStr"/>
+      <c r="FZ2" t="inlineStr"/>
+      <c r="GA2" t="inlineStr"/>
+      <c r="GB2" t="inlineStr"/>
+      <c r="GC2" t="inlineStr"/>
+      <c r="GD2" t="inlineStr"/>
+      <c r="GE2" t="inlineStr"/>
+      <c r="GF2" t="inlineStr"/>
+      <c r="GG2" t="inlineStr"/>
+      <c r="GH2" t="inlineStr"/>
+      <c r="GI2" t="inlineStr"/>
+      <c r="GJ2" t="inlineStr"/>
+      <c r="GK2" t="inlineStr"/>
+      <c r="GL2" t="inlineStr"/>
+      <c r="GM2" t="inlineStr"/>
+      <c r="GN2" t="inlineStr"/>
+      <c r="GO2" t="inlineStr"/>
+      <c r="GP2" t="inlineStr"/>
+      <c r="GQ2" t="inlineStr"/>
+      <c r="GR2" t="inlineStr"/>
+      <c r="GS2" t="inlineStr"/>
+      <c r="GT2" t="inlineStr"/>
+      <c r="GU2" t="inlineStr"/>
+      <c r="GV2" t="inlineStr"/>
+      <c r="GW2" t="inlineStr"/>
+      <c r="GX2" t="inlineStr"/>
+      <c r="GY2" t="inlineStr"/>
+      <c r="GZ2" t="inlineStr"/>
+      <c r="HA2" t="inlineStr"/>
+      <c r="HB2" t="inlineStr"/>
+      <c r="HC2" t="inlineStr"/>
+      <c r="HD2" t="inlineStr"/>
+      <c r="HE2" t="inlineStr"/>
+      <c r="HF2" t="inlineStr"/>
+      <c r="HG2" t="inlineStr"/>
+      <c r="HH2" t="inlineStr"/>
+      <c r="HI2" t="inlineStr"/>
+      <c r="HJ2" t="inlineStr"/>
+      <c r="HK2" t="inlineStr"/>
+      <c r="HL2" t="inlineStr"/>
+      <c r="HM2" t="inlineStr"/>
+      <c r="HN2" t="inlineStr"/>
+      <c r="HO2" t="inlineStr"/>
+      <c r="HP2" t="inlineStr"/>
+      <c r="HQ2" t="inlineStr"/>
+      <c r="HR2" t="inlineStr"/>
+      <c r="HS2" t="inlineStr"/>
+      <c r="HT2" t="inlineStr"/>
+      <c r="HU2" t="inlineStr"/>
+      <c r="HV2" t="inlineStr"/>
+      <c r="HW2" t="inlineStr"/>
+      <c r="HX2" t="inlineStr"/>
+      <c r="HY2" t="inlineStr"/>
+      <c r="HZ2" t="inlineStr"/>
+      <c r="IA2" t="inlineStr"/>
+      <c r="IB2" t="inlineStr"/>
+      <c r="IC2" t="inlineStr"/>
+      <c r="ID2" t="inlineStr"/>
+      <c r="IE2" t="inlineStr"/>
+      <c r="IF2" t="inlineStr"/>
+      <c r="IG2" t="inlineStr"/>
+      <c r="IH2" t="inlineStr"/>
+      <c r="II2" t="inlineStr"/>
+      <c r="IJ2" t="inlineStr"/>
+      <c r="IK2" t="inlineStr"/>
+      <c r="IL2" t="inlineStr"/>
+      <c r="IM2" t="inlineStr"/>
+      <c r="IN2" t="inlineStr"/>
+      <c r="IO2" t="inlineStr"/>
+      <c r="IP2" t="inlineStr"/>
+      <c r="IQ2" t="inlineStr"/>
+      <c r="IR2" t="inlineStr"/>
+      <c r="IS2" t="inlineStr"/>
+      <c r="IT2" t="inlineStr"/>
+      <c r="IU2" t="inlineStr"/>
+      <c r="IV2" t="inlineStr"/>
+      <c r="IW2" t="inlineStr"/>
+      <c r="IX2" t="inlineStr"/>
+      <c r="IY2" t="inlineStr"/>
+      <c r="IZ2" t="inlineStr"/>
+      <c r="JA2" t="inlineStr"/>
+      <c r="JB2" t="inlineStr"/>
+      <c r="JC2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1112,6 +2324,208 @@
       <c r="BI3" t="n">
         <v>0.1212439507557961</v>
       </c>
+      <c r="BJ3" t="inlineStr"/>
+      <c r="BK3" t="inlineStr"/>
+      <c r="BL3" t="inlineStr"/>
+      <c r="BM3" t="inlineStr"/>
+      <c r="BN3" t="inlineStr"/>
+      <c r="BO3" t="inlineStr"/>
+      <c r="BP3" t="inlineStr"/>
+      <c r="BQ3" t="inlineStr"/>
+      <c r="BR3" t="inlineStr"/>
+      <c r="BS3" t="inlineStr"/>
+      <c r="BT3" t="inlineStr"/>
+      <c r="BU3" t="inlineStr"/>
+      <c r="BV3" t="inlineStr"/>
+      <c r="BW3" t="inlineStr"/>
+      <c r="BX3" t="inlineStr"/>
+      <c r="BY3" t="inlineStr"/>
+      <c r="BZ3" t="inlineStr"/>
+      <c r="CA3" t="inlineStr"/>
+      <c r="CB3" t="inlineStr"/>
+      <c r="CC3" t="inlineStr"/>
+      <c r="CD3" t="inlineStr"/>
+      <c r="CE3" t="inlineStr"/>
+      <c r="CF3" t="inlineStr"/>
+      <c r="CG3" t="inlineStr"/>
+      <c r="CH3" t="inlineStr"/>
+      <c r="CI3" t="inlineStr"/>
+      <c r="CJ3" t="inlineStr"/>
+      <c r="CK3" t="inlineStr"/>
+      <c r="CL3" t="inlineStr"/>
+      <c r="CM3" t="inlineStr"/>
+      <c r="CN3" t="inlineStr"/>
+      <c r="CO3" t="inlineStr"/>
+      <c r="CP3" t="inlineStr"/>
+      <c r="CQ3" t="inlineStr"/>
+      <c r="CR3" t="inlineStr"/>
+      <c r="CS3" t="inlineStr"/>
+      <c r="CT3" t="inlineStr"/>
+      <c r="CU3" t="inlineStr"/>
+      <c r="CV3" t="inlineStr"/>
+      <c r="CW3" t="inlineStr"/>
+      <c r="CX3" t="inlineStr"/>
+      <c r="CY3" t="inlineStr"/>
+      <c r="CZ3" t="inlineStr"/>
+      <c r="DA3" t="inlineStr"/>
+      <c r="DB3" t="inlineStr"/>
+      <c r="DC3" t="inlineStr"/>
+      <c r="DD3" t="inlineStr"/>
+      <c r="DE3" t="inlineStr"/>
+      <c r="DF3" t="inlineStr"/>
+      <c r="DG3" t="inlineStr"/>
+      <c r="DH3" t="inlineStr"/>
+      <c r="DI3" t="inlineStr"/>
+      <c r="DJ3" t="inlineStr"/>
+      <c r="DK3" t="inlineStr"/>
+      <c r="DL3" t="inlineStr"/>
+      <c r="DM3" t="inlineStr"/>
+      <c r="DN3" t="inlineStr"/>
+      <c r="DO3" t="inlineStr"/>
+      <c r="DP3" t="inlineStr"/>
+      <c r="DQ3" t="inlineStr"/>
+      <c r="DR3" t="inlineStr"/>
+      <c r="DS3" t="inlineStr"/>
+      <c r="DT3" t="inlineStr"/>
+      <c r="DU3" t="inlineStr"/>
+      <c r="DV3" t="inlineStr"/>
+      <c r="DW3" t="inlineStr"/>
+      <c r="DX3" t="inlineStr"/>
+      <c r="DY3" t="inlineStr"/>
+      <c r="DZ3" t="inlineStr"/>
+      <c r="EA3" t="inlineStr"/>
+      <c r="EB3" t="inlineStr"/>
+      <c r="EC3" t="inlineStr"/>
+      <c r="ED3" t="inlineStr"/>
+      <c r="EE3" t="inlineStr"/>
+      <c r="EF3" t="inlineStr"/>
+      <c r="EG3" t="inlineStr"/>
+      <c r="EH3" t="inlineStr"/>
+      <c r="EI3" t="inlineStr"/>
+      <c r="EJ3" t="inlineStr"/>
+      <c r="EK3" t="inlineStr"/>
+      <c r="EL3" t="inlineStr"/>
+      <c r="EM3" t="inlineStr"/>
+      <c r="EN3" t="inlineStr"/>
+      <c r="EO3" t="inlineStr"/>
+      <c r="EP3" t="inlineStr"/>
+      <c r="EQ3" t="inlineStr"/>
+      <c r="ER3" t="inlineStr"/>
+      <c r="ES3" t="inlineStr"/>
+      <c r="ET3" t="inlineStr"/>
+      <c r="EU3" t="inlineStr"/>
+      <c r="EV3" t="inlineStr"/>
+      <c r="EW3" t="inlineStr"/>
+      <c r="EX3" t="inlineStr"/>
+      <c r="EY3" t="inlineStr"/>
+      <c r="EZ3" t="inlineStr"/>
+      <c r="FA3" t="inlineStr"/>
+      <c r="FB3" t="inlineStr"/>
+      <c r="FC3" t="inlineStr"/>
+      <c r="FD3" t="inlineStr"/>
+      <c r="FE3" t="inlineStr"/>
+      <c r="FF3" t="inlineStr"/>
+      <c r="FG3" t="inlineStr"/>
+      <c r="FH3" t="inlineStr"/>
+      <c r="FI3" t="inlineStr"/>
+      <c r="FJ3" t="inlineStr"/>
+      <c r="FK3" t="inlineStr"/>
+      <c r="FL3" t="inlineStr"/>
+      <c r="FM3" t="inlineStr"/>
+      <c r="FN3" t="inlineStr"/>
+      <c r="FO3" t="inlineStr"/>
+      <c r="FP3" t="inlineStr"/>
+      <c r="FQ3" t="inlineStr"/>
+      <c r="FR3" t="inlineStr"/>
+      <c r="FS3" t="inlineStr"/>
+      <c r="FT3" t="inlineStr"/>
+      <c r="FU3" t="inlineStr"/>
+      <c r="FV3" t="inlineStr"/>
+      <c r="FW3" t="inlineStr"/>
+      <c r="FX3" t="inlineStr"/>
+      <c r="FY3" t="inlineStr"/>
+      <c r="FZ3" t="inlineStr"/>
+      <c r="GA3" t="inlineStr"/>
+      <c r="GB3" t="inlineStr"/>
+      <c r="GC3" t="inlineStr"/>
+      <c r="GD3" t="inlineStr"/>
+      <c r="GE3" t="inlineStr"/>
+      <c r="GF3" t="inlineStr"/>
+      <c r="GG3" t="inlineStr"/>
+      <c r="GH3" t="inlineStr"/>
+      <c r="GI3" t="inlineStr"/>
+      <c r="GJ3" t="inlineStr"/>
+      <c r="GK3" t="inlineStr"/>
+      <c r="GL3" t="inlineStr"/>
+      <c r="GM3" t="inlineStr"/>
+      <c r="GN3" t="inlineStr"/>
+      <c r="GO3" t="inlineStr"/>
+      <c r="GP3" t="inlineStr"/>
+      <c r="GQ3" t="inlineStr"/>
+      <c r="GR3" t="inlineStr"/>
+      <c r="GS3" t="inlineStr"/>
+      <c r="GT3" t="inlineStr"/>
+      <c r="GU3" t="inlineStr"/>
+      <c r="GV3" t="inlineStr"/>
+      <c r="GW3" t="inlineStr"/>
+      <c r="GX3" t="inlineStr"/>
+      <c r="GY3" t="inlineStr"/>
+      <c r="GZ3" t="inlineStr"/>
+      <c r="HA3" t="inlineStr"/>
+      <c r="HB3" t="inlineStr"/>
+      <c r="HC3" t="inlineStr"/>
+      <c r="HD3" t="inlineStr"/>
+      <c r="HE3" t="inlineStr"/>
+      <c r="HF3" t="inlineStr"/>
+      <c r="HG3" t="inlineStr"/>
+      <c r="HH3" t="inlineStr"/>
+      <c r="HI3" t="inlineStr"/>
+      <c r="HJ3" t="inlineStr"/>
+      <c r="HK3" t="inlineStr"/>
+      <c r="HL3" t="inlineStr"/>
+      <c r="HM3" t="inlineStr"/>
+      <c r="HN3" t="inlineStr"/>
+      <c r="HO3" t="inlineStr"/>
+      <c r="HP3" t="inlineStr"/>
+      <c r="HQ3" t="inlineStr"/>
+      <c r="HR3" t="inlineStr"/>
+      <c r="HS3" t="inlineStr"/>
+      <c r="HT3" t="inlineStr"/>
+      <c r="HU3" t="inlineStr"/>
+      <c r="HV3" t="inlineStr"/>
+      <c r="HW3" t="inlineStr"/>
+      <c r="HX3" t="inlineStr"/>
+      <c r="HY3" t="inlineStr"/>
+      <c r="HZ3" t="inlineStr"/>
+      <c r="IA3" t="inlineStr"/>
+      <c r="IB3" t="inlineStr"/>
+      <c r="IC3" t="inlineStr"/>
+      <c r="ID3" t="inlineStr"/>
+      <c r="IE3" t="inlineStr"/>
+      <c r="IF3" t="inlineStr"/>
+      <c r="IG3" t="inlineStr"/>
+      <c r="IH3" t="inlineStr"/>
+      <c r="II3" t="inlineStr"/>
+      <c r="IJ3" t="inlineStr"/>
+      <c r="IK3" t="inlineStr"/>
+      <c r="IL3" t="inlineStr"/>
+      <c r="IM3" t="inlineStr"/>
+      <c r="IN3" t="inlineStr"/>
+      <c r="IO3" t="inlineStr"/>
+      <c r="IP3" t="inlineStr"/>
+      <c r="IQ3" t="inlineStr"/>
+      <c r="IR3" t="inlineStr"/>
+      <c r="IS3" t="inlineStr"/>
+      <c r="IT3" t="inlineStr"/>
+      <c r="IU3" t="inlineStr"/>
+      <c r="IV3" t="inlineStr"/>
+      <c r="IW3" t="inlineStr"/>
+      <c r="IX3" t="inlineStr"/>
+      <c r="IY3" t="inlineStr"/>
+      <c r="IZ3" t="inlineStr"/>
+      <c r="JA3" t="inlineStr"/>
+      <c r="JB3" t="inlineStr"/>
+      <c r="JC3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1301,6 +2715,208 @@
       <c r="BI4" t="n">
         <v>0.1212439507557961</v>
       </c>
+      <c r="BJ4" t="inlineStr"/>
+      <c r="BK4" t="inlineStr"/>
+      <c r="BL4" t="inlineStr"/>
+      <c r="BM4" t="inlineStr"/>
+      <c r="BN4" t="inlineStr"/>
+      <c r="BO4" t="inlineStr"/>
+      <c r="BP4" t="inlineStr"/>
+      <c r="BQ4" t="inlineStr"/>
+      <c r="BR4" t="inlineStr"/>
+      <c r="BS4" t="inlineStr"/>
+      <c r="BT4" t="inlineStr"/>
+      <c r="BU4" t="inlineStr"/>
+      <c r="BV4" t="inlineStr"/>
+      <c r="BW4" t="inlineStr"/>
+      <c r="BX4" t="inlineStr"/>
+      <c r="BY4" t="inlineStr"/>
+      <c r="BZ4" t="inlineStr"/>
+      <c r="CA4" t="inlineStr"/>
+      <c r="CB4" t="inlineStr"/>
+      <c r="CC4" t="inlineStr"/>
+      <c r="CD4" t="inlineStr"/>
+      <c r="CE4" t="inlineStr"/>
+      <c r="CF4" t="inlineStr"/>
+      <c r="CG4" t="inlineStr"/>
+      <c r="CH4" t="inlineStr"/>
+      <c r="CI4" t="inlineStr"/>
+      <c r="CJ4" t="inlineStr"/>
+      <c r="CK4" t="inlineStr"/>
+      <c r="CL4" t="inlineStr"/>
+      <c r="CM4" t="inlineStr"/>
+      <c r="CN4" t="inlineStr"/>
+      <c r="CO4" t="inlineStr"/>
+      <c r="CP4" t="inlineStr"/>
+      <c r="CQ4" t="inlineStr"/>
+      <c r="CR4" t="inlineStr"/>
+      <c r="CS4" t="inlineStr"/>
+      <c r="CT4" t="inlineStr"/>
+      <c r="CU4" t="inlineStr"/>
+      <c r="CV4" t="inlineStr"/>
+      <c r="CW4" t="inlineStr"/>
+      <c r="CX4" t="inlineStr"/>
+      <c r="CY4" t="inlineStr"/>
+      <c r="CZ4" t="inlineStr"/>
+      <c r="DA4" t="inlineStr"/>
+      <c r="DB4" t="inlineStr"/>
+      <c r="DC4" t="inlineStr"/>
+      <c r="DD4" t="inlineStr"/>
+      <c r="DE4" t="inlineStr"/>
+      <c r="DF4" t="inlineStr"/>
+      <c r="DG4" t="inlineStr"/>
+      <c r="DH4" t="inlineStr"/>
+      <c r="DI4" t="inlineStr"/>
+      <c r="DJ4" t="inlineStr"/>
+      <c r="DK4" t="inlineStr"/>
+      <c r="DL4" t="inlineStr"/>
+      <c r="DM4" t="inlineStr"/>
+      <c r="DN4" t="inlineStr"/>
+      <c r="DO4" t="inlineStr"/>
+      <c r="DP4" t="inlineStr"/>
+      <c r="DQ4" t="inlineStr"/>
+      <c r="DR4" t="inlineStr"/>
+      <c r="DS4" t="inlineStr"/>
+      <c r="DT4" t="inlineStr"/>
+      <c r="DU4" t="inlineStr"/>
+      <c r="DV4" t="inlineStr"/>
+      <c r="DW4" t="inlineStr"/>
+      <c r="DX4" t="inlineStr"/>
+      <c r="DY4" t="inlineStr"/>
+      <c r="DZ4" t="inlineStr"/>
+      <c r="EA4" t="inlineStr"/>
+      <c r="EB4" t="inlineStr"/>
+      <c r="EC4" t="inlineStr"/>
+      <c r="ED4" t="inlineStr"/>
+      <c r="EE4" t="inlineStr"/>
+      <c r="EF4" t="inlineStr"/>
+      <c r="EG4" t="inlineStr"/>
+      <c r="EH4" t="inlineStr"/>
+      <c r="EI4" t="inlineStr"/>
+      <c r="EJ4" t="inlineStr"/>
+      <c r="EK4" t="inlineStr"/>
+      <c r="EL4" t="inlineStr"/>
+      <c r="EM4" t="inlineStr"/>
+      <c r="EN4" t="inlineStr"/>
+      <c r="EO4" t="inlineStr"/>
+      <c r="EP4" t="inlineStr"/>
+      <c r="EQ4" t="inlineStr"/>
+      <c r="ER4" t="inlineStr"/>
+      <c r="ES4" t="inlineStr"/>
+      <c r="ET4" t="inlineStr"/>
+      <c r="EU4" t="inlineStr"/>
+      <c r="EV4" t="inlineStr"/>
+      <c r="EW4" t="inlineStr"/>
+      <c r="EX4" t="inlineStr"/>
+      <c r="EY4" t="inlineStr"/>
+      <c r="EZ4" t="inlineStr"/>
+      <c r="FA4" t="inlineStr"/>
+      <c r="FB4" t="inlineStr"/>
+      <c r="FC4" t="inlineStr"/>
+      <c r="FD4" t="inlineStr"/>
+      <c r="FE4" t="inlineStr"/>
+      <c r="FF4" t="inlineStr"/>
+      <c r="FG4" t="inlineStr"/>
+      <c r="FH4" t="inlineStr"/>
+      <c r="FI4" t="inlineStr"/>
+      <c r="FJ4" t="inlineStr"/>
+      <c r="FK4" t="inlineStr"/>
+      <c r="FL4" t="inlineStr"/>
+      <c r="FM4" t="inlineStr"/>
+      <c r="FN4" t="inlineStr"/>
+      <c r="FO4" t="inlineStr"/>
+      <c r="FP4" t="inlineStr"/>
+      <c r="FQ4" t="inlineStr"/>
+      <c r="FR4" t="inlineStr"/>
+      <c r="FS4" t="inlineStr"/>
+      <c r="FT4" t="inlineStr"/>
+      <c r="FU4" t="inlineStr"/>
+      <c r="FV4" t="inlineStr"/>
+      <c r="FW4" t="inlineStr"/>
+      <c r="FX4" t="inlineStr"/>
+      <c r="FY4" t="inlineStr"/>
+      <c r="FZ4" t="inlineStr"/>
+      <c r="GA4" t="inlineStr"/>
+      <c r="GB4" t="inlineStr"/>
+      <c r="GC4" t="inlineStr"/>
+      <c r="GD4" t="inlineStr"/>
+      <c r="GE4" t="inlineStr"/>
+      <c r="GF4" t="inlineStr"/>
+      <c r="GG4" t="inlineStr"/>
+      <c r="GH4" t="inlineStr"/>
+      <c r="GI4" t="inlineStr"/>
+      <c r="GJ4" t="inlineStr"/>
+      <c r="GK4" t="inlineStr"/>
+      <c r="GL4" t="inlineStr"/>
+      <c r="GM4" t="inlineStr"/>
+      <c r="GN4" t="inlineStr"/>
+      <c r="GO4" t="inlineStr"/>
+      <c r="GP4" t="inlineStr"/>
+      <c r="GQ4" t="inlineStr"/>
+      <c r="GR4" t="inlineStr"/>
+      <c r="GS4" t="inlineStr"/>
+      <c r="GT4" t="inlineStr"/>
+      <c r="GU4" t="inlineStr"/>
+      <c r="GV4" t="inlineStr"/>
+      <c r="GW4" t="inlineStr"/>
+      <c r="GX4" t="inlineStr"/>
+      <c r="GY4" t="inlineStr"/>
+      <c r="GZ4" t="inlineStr"/>
+      <c r="HA4" t="inlineStr"/>
+      <c r="HB4" t="inlineStr"/>
+      <c r="HC4" t="inlineStr"/>
+      <c r="HD4" t="inlineStr"/>
+      <c r="HE4" t="inlineStr"/>
+      <c r="HF4" t="inlineStr"/>
+      <c r="HG4" t="inlineStr"/>
+      <c r="HH4" t="inlineStr"/>
+      <c r="HI4" t="inlineStr"/>
+      <c r="HJ4" t="inlineStr"/>
+      <c r="HK4" t="inlineStr"/>
+      <c r="HL4" t="inlineStr"/>
+      <c r="HM4" t="inlineStr"/>
+      <c r="HN4" t="inlineStr"/>
+      <c r="HO4" t="inlineStr"/>
+      <c r="HP4" t="inlineStr"/>
+      <c r="HQ4" t="inlineStr"/>
+      <c r="HR4" t="inlineStr"/>
+      <c r="HS4" t="inlineStr"/>
+      <c r="HT4" t="inlineStr"/>
+      <c r="HU4" t="inlineStr"/>
+      <c r="HV4" t="inlineStr"/>
+      <c r="HW4" t="inlineStr"/>
+      <c r="HX4" t="inlineStr"/>
+      <c r="HY4" t="inlineStr"/>
+      <c r="HZ4" t="inlineStr"/>
+      <c r="IA4" t="inlineStr"/>
+      <c r="IB4" t="inlineStr"/>
+      <c r="IC4" t="inlineStr"/>
+      <c r="ID4" t="inlineStr"/>
+      <c r="IE4" t="inlineStr"/>
+      <c r="IF4" t="inlineStr"/>
+      <c r="IG4" t="inlineStr"/>
+      <c r="IH4" t="inlineStr"/>
+      <c r="II4" t="inlineStr"/>
+      <c r="IJ4" t="inlineStr"/>
+      <c r="IK4" t="inlineStr"/>
+      <c r="IL4" t="inlineStr"/>
+      <c r="IM4" t="inlineStr"/>
+      <c r="IN4" t="inlineStr"/>
+      <c r="IO4" t="inlineStr"/>
+      <c r="IP4" t="inlineStr"/>
+      <c r="IQ4" t="inlineStr"/>
+      <c r="IR4" t="inlineStr"/>
+      <c r="IS4" t="inlineStr"/>
+      <c r="IT4" t="inlineStr"/>
+      <c r="IU4" t="inlineStr"/>
+      <c r="IV4" t="inlineStr"/>
+      <c r="IW4" t="inlineStr"/>
+      <c r="IX4" t="inlineStr"/>
+      <c r="IY4" t="inlineStr"/>
+      <c r="IZ4" t="inlineStr"/>
+      <c r="JA4" t="inlineStr"/>
+      <c r="JB4" t="inlineStr"/>
+      <c r="JC4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1490,6 +3106,208 @@
       <c r="BI5" t="n">
         <v>0.1212439507557961</v>
       </c>
+      <c r="BJ5" t="inlineStr"/>
+      <c r="BK5" t="inlineStr"/>
+      <c r="BL5" t="inlineStr"/>
+      <c r="BM5" t="inlineStr"/>
+      <c r="BN5" t="inlineStr"/>
+      <c r="BO5" t="inlineStr"/>
+      <c r="BP5" t="inlineStr"/>
+      <c r="BQ5" t="inlineStr"/>
+      <c r="BR5" t="inlineStr"/>
+      <c r="BS5" t="inlineStr"/>
+      <c r="BT5" t="inlineStr"/>
+      <c r="BU5" t="inlineStr"/>
+      <c r="BV5" t="inlineStr"/>
+      <c r="BW5" t="inlineStr"/>
+      <c r="BX5" t="inlineStr"/>
+      <c r="BY5" t="inlineStr"/>
+      <c r="BZ5" t="inlineStr"/>
+      <c r="CA5" t="inlineStr"/>
+      <c r="CB5" t="inlineStr"/>
+      <c r="CC5" t="inlineStr"/>
+      <c r="CD5" t="inlineStr"/>
+      <c r="CE5" t="inlineStr"/>
+      <c r="CF5" t="inlineStr"/>
+      <c r="CG5" t="inlineStr"/>
+      <c r="CH5" t="inlineStr"/>
+      <c r="CI5" t="inlineStr"/>
+      <c r="CJ5" t="inlineStr"/>
+      <c r="CK5" t="inlineStr"/>
+      <c r="CL5" t="inlineStr"/>
+      <c r="CM5" t="inlineStr"/>
+      <c r="CN5" t="inlineStr"/>
+      <c r="CO5" t="inlineStr"/>
+      <c r="CP5" t="inlineStr"/>
+      <c r="CQ5" t="inlineStr"/>
+      <c r="CR5" t="inlineStr"/>
+      <c r="CS5" t="inlineStr"/>
+      <c r="CT5" t="inlineStr"/>
+      <c r="CU5" t="inlineStr"/>
+      <c r="CV5" t="inlineStr"/>
+      <c r="CW5" t="inlineStr"/>
+      <c r="CX5" t="inlineStr"/>
+      <c r="CY5" t="inlineStr"/>
+      <c r="CZ5" t="inlineStr"/>
+      <c r="DA5" t="inlineStr"/>
+      <c r="DB5" t="inlineStr"/>
+      <c r="DC5" t="inlineStr"/>
+      <c r="DD5" t="inlineStr"/>
+      <c r="DE5" t="inlineStr"/>
+      <c r="DF5" t="inlineStr"/>
+      <c r="DG5" t="inlineStr"/>
+      <c r="DH5" t="inlineStr"/>
+      <c r="DI5" t="inlineStr"/>
+      <c r="DJ5" t="inlineStr"/>
+      <c r="DK5" t="inlineStr"/>
+      <c r="DL5" t="inlineStr"/>
+      <c r="DM5" t="inlineStr"/>
+      <c r="DN5" t="inlineStr"/>
+      <c r="DO5" t="inlineStr"/>
+      <c r="DP5" t="inlineStr"/>
+      <c r="DQ5" t="inlineStr"/>
+      <c r="DR5" t="inlineStr"/>
+      <c r="DS5" t="inlineStr"/>
+      <c r="DT5" t="inlineStr"/>
+      <c r="DU5" t="inlineStr"/>
+      <c r="DV5" t="inlineStr"/>
+      <c r="DW5" t="inlineStr"/>
+      <c r="DX5" t="inlineStr"/>
+      <c r="DY5" t="inlineStr"/>
+      <c r="DZ5" t="inlineStr"/>
+      <c r="EA5" t="inlineStr"/>
+      <c r="EB5" t="inlineStr"/>
+      <c r="EC5" t="inlineStr"/>
+      <c r="ED5" t="inlineStr"/>
+      <c r="EE5" t="inlineStr"/>
+      <c r="EF5" t="inlineStr"/>
+      <c r="EG5" t="inlineStr"/>
+      <c r="EH5" t="inlineStr"/>
+      <c r="EI5" t="inlineStr"/>
+      <c r="EJ5" t="inlineStr"/>
+      <c r="EK5" t="inlineStr"/>
+      <c r="EL5" t="inlineStr"/>
+      <c r="EM5" t="inlineStr"/>
+      <c r="EN5" t="inlineStr"/>
+      <c r="EO5" t="inlineStr"/>
+      <c r="EP5" t="inlineStr"/>
+      <c r="EQ5" t="inlineStr"/>
+      <c r="ER5" t="inlineStr"/>
+      <c r="ES5" t="inlineStr"/>
+      <c r="ET5" t="inlineStr"/>
+      <c r="EU5" t="inlineStr"/>
+      <c r="EV5" t="inlineStr"/>
+      <c r="EW5" t="inlineStr"/>
+      <c r="EX5" t="inlineStr"/>
+      <c r="EY5" t="inlineStr"/>
+      <c r="EZ5" t="inlineStr"/>
+      <c r="FA5" t="inlineStr"/>
+      <c r="FB5" t="inlineStr"/>
+      <c r="FC5" t="inlineStr"/>
+      <c r="FD5" t="inlineStr"/>
+      <c r="FE5" t="inlineStr"/>
+      <c r="FF5" t="inlineStr"/>
+      <c r="FG5" t="inlineStr"/>
+      <c r="FH5" t="inlineStr"/>
+      <c r="FI5" t="inlineStr"/>
+      <c r="FJ5" t="inlineStr"/>
+      <c r="FK5" t="inlineStr"/>
+      <c r="FL5" t="inlineStr"/>
+      <c r="FM5" t="inlineStr"/>
+      <c r="FN5" t="inlineStr"/>
+      <c r="FO5" t="inlineStr"/>
+      <c r="FP5" t="inlineStr"/>
+      <c r="FQ5" t="inlineStr"/>
+      <c r="FR5" t="inlineStr"/>
+      <c r="FS5" t="inlineStr"/>
+      <c r="FT5" t="inlineStr"/>
+      <c r="FU5" t="inlineStr"/>
+      <c r="FV5" t="inlineStr"/>
+      <c r="FW5" t="inlineStr"/>
+      <c r="FX5" t="inlineStr"/>
+      <c r="FY5" t="inlineStr"/>
+      <c r="FZ5" t="inlineStr"/>
+      <c r="GA5" t="inlineStr"/>
+      <c r="GB5" t="inlineStr"/>
+      <c r="GC5" t="inlineStr"/>
+      <c r="GD5" t="inlineStr"/>
+      <c r="GE5" t="inlineStr"/>
+      <c r="GF5" t="inlineStr"/>
+      <c r="GG5" t="inlineStr"/>
+      <c r="GH5" t="inlineStr"/>
+      <c r="GI5" t="inlineStr"/>
+      <c r="GJ5" t="inlineStr"/>
+      <c r="GK5" t="inlineStr"/>
+      <c r="GL5" t="inlineStr"/>
+      <c r="GM5" t="inlineStr"/>
+      <c r="GN5" t="inlineStr"/>
+      <c r="GO5" t="inlineStr"/>
+      <c r="GP5" t="inlineStr"/>
+      <c r="GQ5" t="inlineStr"/>
+      <c r="GR5" t="inlineStr"/>
+      <c r="GS5" t="inlineStr"/>
+      <c r="GT5" t="inlineStr"/>
+      <c r="GU5" t="inlineStr"/>
+      <c r="GV5" t="inlineStr"/>
+      <c r="GW5" t="inlineStr"/>
+      <c r="GX5" t="inlineStr"/>
+      <c r="GY5" t="inlineStr"/>
+      <c r="GZ5" t="inlineStr"/>
+      <c r="HA5" t="inlineStr"/>
+      <c r="HB5" t="inlineStr"/>
+      <c r="HC5" t="inlineStr"/>
+      <c r="HD5" t="inlineStr"/>
+      <c r="HE5" t="inlineStr"/>
+      <c r="HF5" t="inlineStr"/>
+      <c r="HG5" t="inlineStr"/>
+      <c r="HH5" t="inlineStr"/>
+      <c r="HI5" t="inlineStr"/>
+      <c r="HJ5" t="inlineStr"/>
+      <c r="HK5" t="inlineStr"/>
+      <c r="HL5" t="inlineStr"/>
+      <c r="HM5" t="inlineStr"/>
+      <c r="HN5" t="inlineStr"/>
+      <c r="HO5" t="inlineStr"/>
+      <c r="HP5" t="inlineStr"/>
+      <c r="HQ5" t="inlineStr"/>
+      <c r="HR5" t="inlineStr"/>
+      <c r="HS5" t="inlineStr"/>
+      <c r="HT5" t="inlineStr"/>
+      <c r="HU5" t="inlineStr"/>
+      <c r="HV5" t="inlineStr"/>
+      <c r="HW5" t="inlineStr"/>
+      <c r="HX5" t="inlineStr"/>
+      <c r="HY5" t="inlineStr"/>
+      <c r="HZ5" t="inlineStr"/>
+      <c r="IA5" t="inlineStr"/>
+      <c r="IB5" t="inlineStr"/>
+      <c r="IC5" t="inlineStr"/>
+      <c r="ID5" t="inlineStr"/>
+      <c r="IE5" t="inlineStr"/>
+      <c r="IF5" t="inlineStr"/>
+      <c r="IG5" t="inlineStr"/>
+      <c r="IH5" t="inlineStr"/>
+      <c r="II5" t="inlineStr"/>
+      <c r="IJ5" t="inlineStr"/>
+      <c r="IK5" t="inlineStr"/>
+      <c r="IL5" t="inlineStr"/>
+      <c r="IM5" t="inlineStr"/>
+      <c r="IN5" t="inlineStr"/>
+      <c r="IO5" t="inlineStr"/>
+      <c r="IP5" t="inlineStr"/>
+      <c r="IQ5" t="inlineStr"/>
+      <c r="IR5" t="inlineStr"/>
+      <c r="IS5" t="inlineStr"/>
+      <c r="IT5" t="inlineStr"/>
+      <c r="IU5" t="inlineStr"/>
+      <c r="IV5" t="inlineStr"/>
+      <c r="IW5" t="inlineStr"/>
+      <c r="IX5" t="inlineStr"/>
+      <c r="IY5" t="inlineStr"/>
+      <c r="IZ5" t="inlineStr"/>
+      <c r="JA5" t="inlineStr"/>
+      <c r="JB5" t="inlineStr"/>
+      <c r="JC5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1613,6 +3431,208 @@
       <c r="BG6" t="inlineStr"/>
       <c r="BH6" t="inlineStr"/>
       <c r="BI6" t="inlineStr"/>
+      <c r="BJ6" t="inlineStr"/>
+      <c r="BK6" t="inlineStr"/>
+      <c r="BL6" t="inlineStr"/>
+      <c r="BM6" t="inlineStr"/>
+      <c r="BN6" t="inlineStr"/>
+      <c r="BO6" t="inlineStr"/>
+      <c r="BP6" t="inlineStr"/>
+      <c r="BQ6" t="inlineStr"/>
+      <c r="BR6" t="inlineStr"/>
+      <c r="BS6" t="inlineStr"/>
+      <c r="BT6" t="inlineStr"/>
+      <c r="BU6" t="inlineStr"/>
+      <c r="BV6" t="inlineStr"/>
+      <c r="BW6" t="inlineStr"/>
+      <c r="BX6" t="inlineStr"/>
+      <c r="BY6" t="inlineStr"/>
+      <c r="BZ6" t="inlineStr"/>
+      <c r="CA6" t="inlineStr"/>
+      <c r="CB6" t="inlineStr"/>
+      <c r="CC6" t="inlineStr"/>
+      <c r="CD6" t="inlineStr"/>
+      <c r="CE6" t="inlineStr"/>
+      <c r="CF6" t="inlineStr"/>
+      <c r="CG6" t="inlineStr"/>
+      <c r="CH6" t="inlineStr"/>
+      <c r="CI6" t="inlineStr"/>
+      <c r="CJ6" t="inlineStr"/>
+      <c r="CK6" t="inlineStr"/>
+      <c r="CL6" t="inlineStr"/>
+      <c r="CM6" t="inlineStr"/>
+      <c r="CN6" t="inlineStr"/>
+      <c r="CO6" t="inlineStr"/>
+      <c r="CP6" t="inlineStr"/>
+      <c r="CQ6" t="inlineStr"/>
+      <c r="CR6" t="inlineStr"/>
+      <c r="CS6" t="inlineStr"/>
+      <c r="CT6" t="inlineStr"/>
+      <c r="CU6" t="inlineStr"/>
+      <c r="CV6" t="inlineStr"/>
+      <c r="CW6" t="inlineStr"/>
+      <c r="CX6" t="inlineStr"/>
+      <c r="CY6" t="inlineStr"/>
+      <c r="CZ6" t="inlineStr"/>
+      <c r="DA6" t="inlineStr"/>
+      <c r="DB6" t="inlineStr"/>
+      <c r="DC6" t="inlineStr"/>
+      <c r="DD6" t="inlineStr"/>
+      <c r="DE6" t="inlineStr"/>
+      <c r="DF6" t="inlineStr"/>
+      <c r="DG6" t="inlineStr"/>
+      <c r="DH6" t="inlineStr"/>
+      <c r="DI6" t="inlineStr"/>
+      <c r="DJ6" t="inlineStr"/>
+      <c r="DK6" t="inlineStr"/>
+      <c r="DL6" t="inlineStr"/>
+      <c r="DM6" t="inlineStr"/>
+      <c r="DN6" t="inlineStr"/>
+      <c r="DO6" t="inlineStr"/>
+      <c r="DP6" t="inlineStr"/>
+      <c r="DQ6" t="inlineStr"/>
+      <c r="DR6" t="inlineStr"/>
+      <c r="DS6" t="inlineStr"/>
+      <c r="DT6" t="inlineStr"/>
+      <c r="DU6" t="inlineStr"/>
+      <c r="DV6" t="inlineStr"/>
+      <c r="DW6" t="inlineStr"/>
+      <c r="DX6" t="inlineStr"/>
+      <c r="DY6" t="inlineStr"/>
+      <c r="DZ6" t="inlineStr"/>
+      <c r="EA6" t="inlineStr"/>
+      <c r="EB6" t="inlineStr"/>
+      <c r="EC6" t="inlineStr"/>
+      <c r="ED6" t="inlineStr"/>
+      <c r="EE6" t="inlineStr"/>
+      <c r="EF6" t="inlineStr"/>
+      <c r="EG6" t="inlineStr"/>
+      <c r="EH6" t="inlineStr"/>
+      <c r="EI6" t="inlineStr"/>
+      <c r="EJ6" t="inlineStr"/>
+      <c r="EK6" t="inlineStr"/>
+      <c r="EL6" t="inlineStr"/>
+      <c r="EM6" t="inlineStr"/>
+      <c r="EN6" t="inlineStr"/>
+      <c r="EO6" t="inlineStr"/>
+      <c r="EP6" t="inlineStr"/>
+      <c r="EQ6" t="inlineStr"/>
+      <c r="ER6" t="inlineStr"/>
+      <c r="ES6" t="inlineStr"/>
+      <c r="ET6" t="inlineStr"/>
+      <c r="EU6" t="inlineStr"/>
+      <c r="EV6" t="inlineStr"/>
+      <c r="EW6" t="inlineStr"/>
+      <c r="EX6" t="inlineStr"/>
+      <c r="EY6" t="inlineStr"/>
+      <c r="EZ6" t="inlineStr"/>
+      <c r="FA6" t="inlineStr"/>
+      <c r="FB6" t="inlineStr"/>
+      <c r="FC6" t="inlineStr"/>
+      <c r="FD6" t="inlineStr"/>
+      <c r="FE6" t="inlineStr"/>
+      <c r="FF6" t="inlineStr"/>
+      <c r="FG6" t="inlineStr"/>
+      <c r="FH6" t="inlineStr"/>
+      <c r="FI6" t="inlineStr"/>
+      <c r="FJ6" t="inlineStr"/>
+      <c r="FK6" t="inlineStr"/>
+      <c r="FL6" t="inlineStr"/>
+      <c r="FM6" t="inlineStr"/>
+      <c r="FN6" t="inlineStr"/>
+      <c r="FO6" t="inlineStr"/>
+      <c r="FP6" t="inlineStr"/>
+      <c r="FQ6" t="inlineStr"/>
+      <c r="FR6" t="inlineStr"/>
+      <c r="FS6" t="inlineStr"/>
+      <c r="FT6" t="inlineStr"/>
+      <c r="FU6" t="inlineStr"/>
+      <c r="FV6" t="inlineStr"/>
+      <c r="FW6" t="inlineStr"/>
+      <c r="FX6" t="inlineStr"/>
+      <c r="FY6" t="inlineStr"/>
+      <c r="FZ6" t="inlineStr"/>
+      <c r="GA6" t="inlineStr"/>
+      <c r="GB6" t="inlineStr"/>
+      <c r="GC6" t="inlineStr"/>
+      <c r="GD6" t="inlineStr"/>
+      <c r="GE6" t="inlineStr"/>
+      <c r="GF6" t="inlineStr"/>
+      <c r="GG6" t="inlineStr"/>
+      <c r="GH6" t="inlineStr"/>
+      <c r="GI6" t="inlineStr"/>
+      <c r="GJ6" t="inlineStr"/>
+      <c r="GK6" t="inlineStr"/>
+      <c r="GL6" t="inlineStr"/>
+      <c r="GM6" t="inlineStr"/>
+      <c r="GN6" t="inlineStr"/>
+      <c r="GO6" t="inlineStr"/>
+      <c r="GP6" t="inlineStr"/>
+      <c r="GQ6" t="inlineStr"/>
+      <c r="GR6" t="inlineStr"/>
+      <c r="GS6" t="inlineStr"/>
+      <c r="GT6" t="inlineStr"/>
+      <c r="GU6" t="inlineStr"/>
+      <c r="GV6" t="inlineStr"/>
+      <c r="GW6" t="inlineStr"/>
+      <c r="GX6" t="inlineStr"/>
+      <c r="GY6" t="inlineStr"/>
+      <c r="GZ6" t="inlineStr"/>
+      <c r="HA6" t="inlineStr"/>
+      <c r="HB6" t="inlineStr"/>
+      <c r="HC6" t="inlineStr"/>
+      <c r="HD6" t="inlineStr"/>
+      <c r="HE6" t="inlineStr"/>
+      <c r="HF6" t="inlineStr"/>
+      <c r="HG6" t="inlineStr"/>
+      <c r="HH6" t="inlineStr"/>
+      <c r="HI6" t="inlineStr"/>
+      <c r="HJ6" t="inlineStr"/>
+      <c r="HK6" t="inlineStr"/>
+      <c r="HL6" t="inlineStr"/>
+      <c r="HM6" t="inlineStr"/>
+      <c r="HN6" t="inlineStr"/>
+      <c r="HO6" t="inlineStr"/>
+      <c r="HP6" t="inlineStr"/>
+      <c r="HQ6" t="inlineStr"/>
+      <c r="HR6" t="inlineStr"/>
+      <c r="HS6" t="inlineStr"/>
+      <c r="HT6" t="inlineStr"/>
+      <c r="HU6" t="inlineStr"/>
+      <c r="HV6" t="inlineStr"/>
+      <c r="HW6" t="inlineStr"/>
+      <c r="HX6" t="inlineStr"/>
+      <c r="HY6" t="inlineStr"/>
+      <c r="HZ6" t="inlineStr"/>
+      <c r="IA6" t="inlineStr"/>
+      <c r="IB6" t="inlineStr"/>
+      <c r="IC6" t="inlineStr"/>
+      <c r="ID6" t="inlineStr"/>
+      <c r="IE6" t="inlineStr"/>
+      <c r="IF6" t="inlineStr"/>
+      <c r="IG6" t="inlineStr"/>
+      <c r="IH6" t="inlineStr"/>
+      <c r="II6" t="inlineStr"/>
+      <c r="IJ6" t="inlineStr"/>
+      <c r="IK6" t="inlineStr"/>
+      <c r="IL6" t="inlineStr"/>
+      <c r="IM6" t="inlineStr"/>
+      <c r="IN6" t="inlineStr"/>
+      <c r="IO6" t="inlineStr"/>
+      <c r="IP6" t="inlineStr"/>
+      <c r="IQ6" t="inlineStr"/>
+      <c r="IR6" t="inlineStr"/>
+      <c r="IS6" t="inlineStr"/>
+      <c r="IT6" t="inlineStr"/>
+      <c r="IU6" t="inlineStr"/>
+      <c r="IV6" t="inlineStr"/>
+      <c r="IW6" t="inlineStr"/>
+      <c r="IX6" t="inlineStr"/>
+      <c r="IY6" t="inlineStr"/>
+      <c r="IZ6" t="inlineStr"/>
+      <c r="JA6" t="inlineStr"/>
+      <c r="JB6" t="inlineStr"/>
+      <c r="JC6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1736,6 +3756,208 @@
       <c r="BG7" t="inlineStr"/>
       <c r="BH7" t="inlineStr"/>
       <c r="BI7" t="inlineStr"/>
+      <c r="BJ7" t="inlineStr"/>
+      <c r="BK7" t="inlineStr"/>
+      <c r="BL7" t="inlineStr"/>
+      <c r="BM7" t="inlineStr"/>
+      <c r="BN7" t="inlineStr"/>
+      <c r="BO7" t="inlineStr"/>
+      <c r="BP7" t="inlineStr"/>
+      <c r="BQ7" t="inlineStr"/>
+      <c r="BR7" t="inlineStr"/>
+      <c r="BS7" t="inlineStr"/>
+      <c r="BT7" t="inlineStr"/>
+      <c r="BU7" t="inlineStr"/>
+      <c r="BV7" t="inlineStr"/>
+      <c r="BW7" t="inlineStr"/>
+      <c r="BX7" t="inlineStr"/>
+      <c r="BY7" t="inlineStr"/>
+      <c r="BZ7" t="inlineStr"/>
+      <c r="CA7" t="inlineStr"/>
+      <c r="CB7" t="inlineStr"/>
+      <c r="CC7" t="inlineStr"/>
+      <c r="CD7" t="inlineStr"/>
+      <c r="CE7" t="inlineStr"/>
+      <c r="CF7" t="inlineStr"/>
+      <c r="CG7" t="inlineStr"/>
+      <c r="CH7" t="inlineStr"/>
+      <c r="CI7" t="inlineStr"/>
+      <c r="CJ7" t="inlineStr"/>
+      <c r="CK7" t="inlineStr"/>
+      <c r="CL7" t="inlineStr"/>
+      <c r="CM7" t="inlineStr"/>
+      <c r="CN7" t="inlineStr"/>
+      <c r="CO7" t="inlineStr"/>
+      <c r="CP7" t="inlineStr"/>
+      <c r="CQ7" t="inlineStr"/>
+      <c r="CR7" t="inlineStr"/>
+      <c r="CS7" t="inlineStr"/>
+      <c r="CT7" t="inlineStr"/>
+      <c r="CU7" t="inlineStr"/>
+      <c r="CV7" t="inlineStr"/>
+      <c r="CW7" t="inlineStr"/>
+      <c r="CX7" t="inlineStr"/>
+      <c r="CY7" t="inlineStr"/>
+      <c r="CZ7" t="inlineStr"/>
+      <c r="DA7" t="inlineStr"/>
+      <c r="DB7" t="inlineStr"/>
+      <c r="DC7" t="inlineStr"/>
+      <c r="DD7" t="inlineStr"/>
+      <c r="DE7" t="inlineStr"/>
+      <c r="DF7" t="inlineStr"/>
+      <c r="DG7" t="inlineStr"/>
+      <c r="DH7" t="inlineStr"/>
+      <c r="DI7" t="inlineStr"/>
+      <c r="DJ7" t="inlineStr"/>
+      <c r="DK7" t="inlineStr"/>
+      <c r="DL7" t="inlineStr"/>
+      <c r="DM7" t="inlineStr"/>
+      <c r="DN7" t="inlineStr"/>
+      <c r="DO7" t="inlineStr"/>
+      <c r="DP7" t="inlineStr"/>
+      <c r="DQ7" t="inlineStr"/>
+      <c r="DR7" t="inlineStr"/>
+      <c r="DS7" t="inlineStr"/>
+      <c r="DT7" t="inlineStr"/>
+      <c r="DU7" t="inlineStr"/>
+      <c r="DV7" t="inlineStr"/>
+      <c r="DW7" t="inlineStr"/>
+      <c r="DX7" t="inlineStr"/>
+      <c r="DY7" t="inlineStr"/>
+      <c r="DZ7" t="inlineStr"/>
+      <c r="EA7" t="inlineStr"/>
+      <c r="EB7" t="inlineStr"/>
+      <c r="EC7" t="inlineStr"/>
+      <c r="ED7" t="inlineStr"/>
+      <c r="EE7" t="inlineStr"/>
+      <c r="EF7" t="inlineStr"/>
+      <c r="EG7" t="inlineStr"/>
+      <c r="EH7" t="inlineStr"/>
+      <c r="EI7" t="inlineStr"/>
+      <c r="EJ7" t="inlineStr"/>
+      <c r="EK7" t="inlineStr"/>
+      <c r="EL7" t="inlineStr"/>
+      <c r="EM7" t="inlineStr"/>
+      <c r="EN7" t="inlineStr"/>
+      <c r="EO7" t="inlineStr"/>
+      <c r="EP7" t="inlineStr"/>
+      <c r="EQ7" t="inlineStr"/>
+      <c r="ER7" t="inlineStr"/>
+      <c r="ES7" t="inlineStr"/>
+      <c r="ET7" t="inlineStr"/>
+      <c r="EU7" t="inlineStr"/>
+      <c r="EV7" t="inlineStr"/>
+      <c r="EW7" t="inlineStr"/>
+      <c r="EX7" t="inlineStr"/>
+      <c r="EY7" t="inlineStr"/>
+      <c r="EZ7" t="inlineStr"/>
+      <c r="FA7" t="inlineStr"/>
+      <c r="FB7" t="inlineStr"/>
+      <c r="FC7" t="inlineStr"/>
+      <c r="FD7" t="inlineStr"/>
+      <c r="FE7" t="inlineStr"/>
+      <c r="FF7" t="inlineStr"/>
+      <c r="FG7" t="inlineStr"/>
+      <c r="FH7" t="inlineStr"/>
+      <c r="FI7" t="inlineStr"/>
+      <c r="FJ7" t="inlineStr"/>
+      <c r="FK7" t="inlineStr"/>
+      <c r="FL7" t="inlineStr"/>
+      <c r="FM7" t="inlineStr"/>
+      <c r="FN7" t="inlineStr"/>
+      <c r="FO7" t="inlineStr"/>
+      <c r="FP7" t="inlineStr"/>
+      <c r="FQ7" t="inlineStr"/>
+      <c r="FR7" t="inlineStr"/>
+      <c r="FS7" t="inlineStr"/>
+      <c r="FT7" t="inlineStr"/>
+      <c r="FU7" t="inlineStr"/>
+      <c r="FV7" t="inlineStr"/>
+      <c r="FW7" t="inlineStr"/>
+      <c r="FX7" t="inlineStr"/>
+      <c r="FY7" t="inlineStr"/>
+      <c r="FZ7" t="inlineStr"/>
+      <c r="GA7" t="inlineStr"/>
+      <c r="GB7" t="inlineStr"/>
+      <c r="GC7" t="inlineStr"/>
+      <c r="GD7" t="inlineStr"/>
+      <c r="GE7" t="inlineStr"/>
+      <c r="GF7" t="inlineStr"/>
+      <c r="GG7" t="inlineStr"/>
+      <c r="GH7" t="inlineStr"/>
+      <c r="GI7" t="inlineStr"/>
+      <c r="GJ7" t="inlineStr"/>
+      <c r="GK7" t="inlineStr"/>
+      <c r="GL7" t="inlineStr"/>
+      <c r="GM7" t="inlineStr"/>
+      <c r="GN7" t="inlineStr"/>
+      <c r="GO7" t="inlineStr"/>
+      <c r="GP7" t="inlineStr"/>
+      <c r="GQ7" t="inlineStr"/>
+      <c r="GR7" t="inlineStr"/>
+      <c r="GS7" t="inlineStr"/>
+      <c r="GT7" t="inlineStr"/>
+      <c r="GU7" t="inlineStr"/>
+      <c r="GV7" t="inlineStr"/>
+      <c r="GW7" t="inlineStr"/>
+      <c r="GX7" t="inlineStr"/>
+      <c r="GY7" t="inlineStr"/>
+      <c r="GZ7" t="inlineStr"/>
+      <c r="HA7" t="inlineStr"/>
+      <c r="HB7" t="inlineStr"/>
+      <c r="HC7" t="inlineStr"/>
+      <c r="HD7" t="inlineStr"/>
+      <c r="HE7" t="inlineStr"/>
+      <c r="HF7" t="inlineStr"/>
+      <c r="HG7" t="inlineStr"/>
+      <c r="HH7" t="inlineStr"/>
+      <c r="HI7" t="inlineStr"/>
+      <c r="HJ7" t="inlineStr"/>
+      <c r="HK7" t="inlineStr"/>
+      <c r="HL7" t="inlineStr"/>
+      <c r="HM7" t="inlineStr"/>
+      <c r="HN7" t="inlineStr"/>
+      <c r="HO7" t="inlineStr"/>
+      <c r="HP7" t="inlineStr"/>
+      <c r="HQ7" t="inlineStr"/>
+      <c r="HR7" t="inlineStr"/>
+      <c r="HS7" t="inlineStr"/>
+      <c r="HT7" t="inlineStr"/>
+      <c r="HU7" t="inlineStr"/>
+      <c r="HV7" t="inlineStr"/>
+      <c r="HW7" t="inlineStr"/>
+      <c r="HX7" t="inlineStr"/>
+      <c r="HY7" t="inlineStr"/>
+      <c r="HZ7" t="inlineStr"/>
+      <c r="IA7" t="inlineStr"/>
+      <c r="IB7" t="inlineStr"/>
+      <c r="IC7" t="inlineStr"/>
+      <c r="ID7" t="inlineStr"/>
+      <c r="IE7" t="inlineStr"/>
+      <c r="IF7" t="inlineStr"/>
+      <c r="IG7" t="inlineStr"/>
+      <c r="IH7" t="inlineStr"/>
+      <c r="II7" t="inlineStr"/>
+      <c r="IJ7" t="inlineStr"/>
+      <c r="IK7" t="inlineStr"/>
+      <c r="IL7" t="inlineStr"/>
+      <c r="IM7" t="inlineStr"/>
+      <c r="IN7" t="inlineStr"/>
+      <c r="IO7" t="inlineStr"/>
+      <c r="IP7" t="inlineStr"/>
+      <c r="IQ7" t="inlineStr"/>
+      <c r="IR7" t="inlineStr"/>
+      <c r="IS7" t="inlineStr"/>
+      <c r="IT7" t="inlineStr"/>
+      <c r="IU7" t="inlineStr"/>
+      <c r="IV7" t="inlineStr"/>
+      <c r="IW7" t="inlineStr"/>
+      <c r="IX7" t="inlineStr"/>
+      <c r="IY7" t="inlineStr"/>
+      <c r="IZ7" t="inlineStr"/>
+      <c r="JA7" t="inlineStr"/>
+      <c r="JB7" t="inlineStr"/>
+      <c r="JC7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1869,7 +4091,7 @@
         <v>0</v>
       </c>
       <c r="AQ8" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AR8" t="n">
         <v>0.01269718614916328</v>
@@ -1924,6 +4146,1394 @@
       </c>
       <c r="BI8" t="n">
         <v>0.06162362132781011</v>
+      </c>
+      <c r="BJ8" t="inlineStr"/>
+      <c r="BK8" t="inlineStr"/>
+      <c r="BL8" t="inlineStr"/>
+      <c r="BM8" t="inlineStr"/>
+      <c r="BN8" t="inlineStr"/>
+      <c r="BO8" t="inlineStr"/>
+      <c r="BP8" t="inlineStr"/>
+      <c r="BQ8" t="inlineStr"/>
+      <c r="BR8" t="inlineStr"/>
+      <c r="BS8" t="inlineStr"/>
+      <c r="BT8" t="inlineStr"/>
+      <c r="BU8" t="inlineStr"/>
+      <c r="BV8" t="inlineStr"/>
+      <c r="BW8" t="inlineStr"/>
+      <c r="BX8" t="inlineStr"/>
+      <c r="BY8" t="inlineStr"/>
+      <c r="BZ8" t="inlineStr"/>
+      <c r="CA8" t="inlineStr"/>
+      <c r="CB8" t="inlineStr"/>
+      <c r="CC8" t="inlineStr"/>
+      <c r="CD8" t="inlineStr"/>
+      <c r="CE8" t="inlineStr"/>
+      <c r="CF8" t="inlineStr"/>
+      <c r="CG8" t="inlineStr"/>
+      <c r="CH8" t="inlineStr"/>
+      <c r="CI8" t="inlineStr"/>
+      <c r="CJ8" t="inlineStr"/>
+      <c r="CK8" t="inlineStr"/>
+      <c r="CL8" t="inlineStr"/>
+      <c r="CM8" t="inlineStr"/>
+      <c r="CN8" t="inlineStr"/>
+      <c r="CO8" t="inlineStr"/>
+      <c r="CP8" t="inlineStr"/>
+      <c r="CQ8" t="inlineStr"/>
+      <c r="CR8" t="inlineStr"/>
+      <c r="CS8" t="inlineStr"/>
+      <c r="CT8" t="inlineStr"/>
+      <c r="CU8" t="inlineStr"/>
+      <c r="CV8" t="inlineStr"/>
+      <c r="CW8" t="inlineStr"/>
+      <c r="CX8" t="inlineStr"/>
+      <c r="CY8" t="inlineStr"/>
+      <c r="CZ8" t="inlineStr"/>
+      <c r="DA8" t="inlineStr"/>
+      <c r="DB8" t="inlineStr"/>
+      <c r="DC8" t="inlineStr"/>
+      <c r="DD8" t="inlineStr"/>
+      <c r="DE8" t="inlineStr"/>
+      <c r="DF8" t="inlineStr"/>
+      <c r="DG8" t="inlineStr"/>
+      <c r="DH8" t="inlineStr"/>
+      <c r="DI8" t="inlineStr"/>
+      <c r="DJ8" t="inlineStr"/>
+      <c r="DK8" t="inlineStr"/>
+      <c r="DL8" t="inlineStr"/>
+      <c r="DM8" t="inlineStr"/>
+      <c r="DN8" t="inlineStr"/>
+      <c r="DO8" t="inlineStr"/>
+      <c r="DP8" t="inlineStr"/>
+      <c r="DQ8" t="inlineStr"/>
+      <c r="DR8" t="inlineStr"/>
+      <c r="DS8" t="inlineStr"/>
+      <c r="DT8" t="inlineStr"/>
+      <c r="DU8" t="inlineStr"/>
+      <c r="DV8" t="inlineStr"/>
+      <c r="DW8" t="inlineStr"/>
+      <c r="DX8" t="inlineStr"/>
+      <c r="DY8" t="inlineStr"/>
+      <c r="DZ8" t="inlineStr"/>
+      <c r="EA8" t="inlineStr"/>
+      <c r="EB8" t="inlineStr"/>
+      <c r="EC8" t="inlineStr"/>
+      <c r="ED8" t="inlineStr"/>
+      <c r="EE8" t="inlineStr"/>
+      <c r="EF8" t="inlineStr"/>
+      <c r="EG8" t="inlineStr"/>
+      <c r="EH8" t="inlineStr"/>
+      <c r="EI8" t="inlineStr"/>
+      <c r="EJ8" t="inlineStr"/>
+      <c r="EK8" t="inlineStr"/>
+      <c r="EL8" t="inlineStr"/>
+      <c r="EM8" t="inlineStr"/>
+      <c r="EN8" t="inlineStr"/>
+      <c r="EO8" t="inlineStr"/>
+      <c r="EP8" t="inlineStr"/>
+      <c r="EQ8" t="inlineStr"/>
+      <c r="ER8" t="inlineStr"/>
+      <c r="ES8" t="inlineStr"/>
+      <c r="ET8" t="inlineStr"/>
+      <c r="EU8" t="inlineStr"/>
+      <c r="EV8" t="inlineStr"/>
+      <c r="EW8" t="inlineStr"/>
+      <c r="EX8" t="inlineStr"/>
+      <c r="EY8" t="inlineStr"/>
+      <c r="EZ8" t="inlineStr"/>
+      <c r="FA8" t="inlineStr"/>
+      <c r="FB8" t="inlineStr"/>
+      <c r="FC8" t="inlineStr"/>
+      <c r="FD8" t="inlineStr"/>
+      <c r="FE8" t="inlineStr"/>
+      <c r="FF8" t="inlineStr"/>
+      <c r="FG8" t="inlineStr"/>
+      <c r="FH8" t="inlineStr"/>
+      <c r="FI8" t="inlineStr"/>
+      <c r="FJ8" t="inlineStr"/>
+      <c r="FK8" t="inlineStr"/>
+      <c r="FL8" t="inlineStr"/>
+      <c r="FM8" t="inlineStr"/>
+      <c r="FN8" t="inlineStr"/>
+      <c r="FO8" t="inlineStr"/>
+      <c r="FP8" t="inlineStr"/>
+      <c r="FQ8" t="inlineStr"/>
+      <c r="FR8" t="inlineStr"/>
+      <c r="FS8" t="inlineStr"/>
+      <c r="FT8" t="inlineStr"/>
+      <c r="FU8" t="inlineStr"/>
+      <c r="FV8" t="inlineStr"/>
+      <c r="FW8" t="inlineStr"/>
+      <c r="FX8" t="inlineStr"/>
+      <c r="FY8" t="inlineStr"/>
+      <c r="FZ8" t="inlineStr"/>
+      <c r="GA8" t="inlineStr"/>
+      <c r="GB8" t="inlineStr"/>
+      <c r="GC8" t="inlineStr"/>
+      <c r="GD8" t="inlineStr"/>
+      <c r="GE8" t="inlineStr"/>
+      <c r="GF8" t="inlineStr"/>
+      <c r="GG8" t="inlineStr"/>
+      <c r="GH8" t="inlineStr"/>
+      <c r="GI8" t="inlineStr"/>
+      <c r="GJ8" t="inlineStr"/>
+      <c r="GK8" t="inlineStr"/>
+      <c r="GL8" t="inlineStr"/>
+      <c r="GM8" t="inlineStr"/>
+      <c r="GN8" t="inlineStr"/>
+      <c r="GO8" t="inlineStr"/>
+      <c r="GP8" t="inlineStr"/>
+      <c r="GQ8" t="inlineStr"/>
+      <c r="GR8" t="inlineStr"/>
+      <c r="GS8" t="inlineStr"/>
+      <c r="GT8" t="inlineStr"/>
+      <c r="GU8" t="inlineStr"/>
+      <c r="GV8" t="inlineStr"/>
+      <c r="GW8" t="inlineStr"/>
+      <c r="GX8" t="inlineStr"/>
+      <c r="GY8" t="inlineStr"/>
+      <c r="GZ8" t="inlineStr"/>
+      <c r="HA8" t="inlineStr"/>
+      <c r="HB8" t="inlineStr"/>
+      <c r="HC8" t="inlineStr"/>
+      <c r="HD8" t="inlineStr"/>
+      <c r="HE8" t="inlineStr"/>
+      <c r="HF8" t="inlineStr"/>
+      <c r="HG8" t="inlineStr"/>
+      <c r="HH8" t="inlineStr"/>
+      <c r="HI8" t="inlineStr"/>
+      <c r="HJ8" t="inlineStr"/>
+      <c r="HK8" t="inlineStr"/>
+      <c r="HL8" t="inlineStr"/>
+      <c r="HM8" t="inlineStr"/>
+      <c r="HN8" t="inlineStr"/>
+      <c r="HO8" t="inlineStr"/>
+      <c r="HP8" t="inlineStr"/>
+      <c r="HQ8" t="inlineStr"/>
+      <c r="HR8" t="inlineStr"/>
+      <c r="HS8" t="inlineStr"/>
+      <c r="HT8" t="inlineStr"/>
+      <c r="HU8" t="inlineStr"/>
+      <c r="HV8" t="inlineStr"/>
+      <c r="HW8" t="inlineStr"/>
+      <c r="HX8" t="inlineStr"/>
+      <c r="HY8" t="inlineStr"/>
+      <c r="HZ8" t="inlineStr"/>
+      <c r="IA8" t="inlineStr"/>
+      <c r="IB8" t="inlineStr"/>
+      <c r="IC8" t="inlineStr"/>
+      <c r="ID8" t="inlineStr"/>
+      <c r="IE8" t="inlineStr"/>
+      <c r="IF8" t="inlineStr"/>
+      <c r="IG8" t="inlineStr"/>
+      <c r="IH8" t="inlineStr"/>
+      <c r="II8" t="inlineStr"/>
+      <c r="IJ8" t="inlineStr"/>
+      <c r="IK8" t="inlineStr"/>
+      <c r="IL8" t="inlineStr"/>
+      <c r="IM8" t="inlineStr"/>
+      <c r="IN8" t="inlineStr"/>
+      <c r="IO8" t="inlineStr"/>
+      <c r="IP8" t="inlineStr"/>
+      <c r="IQ8" t="inlineStr"/>
+      <c r="IR8" t="inlineStr"/>
+      <c r="IS8" t="inlineStr"/>
+      <c r="IT8" t="inlineStr"/>
+      <c r="IU8" t="inlineStr"/>
+      <c r="IV8" t="inlineStr"/>
+      <c r="IW8" t="inlineStr"/>
+      <c r="IX8" t="inlineStr"/>
+      <c r="IY8" t="inlineStr"/>
+      <c r="IZ8" t="inlineStr"/>
+      <c r="JA8" t="inlineStr"/>
+      <c r="JB8" t="inlineStr"/>
+      <c r="JC8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-04-15 19:56:28</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>10</v>
+      </c>
+      <c r="C9" t="n">
+        <v>100</v>
+      </c>
+      <c r="D9" t="n">
+        <v>10</v>
+      </c>
+      <c r="E9" t="n">
+        <v>50</v>
+      </c>
+      <c r="F9" t="n">
+        <v>5</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>0.2044303924470618</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0.2704777759813683</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0.2048216012922055</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0.2328183299709716</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0.4472135954999579</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0.4249803482695367</v>
+      </c>
+      <c r="N9" t="n">
+        <v>0.3986680104959187</v>
+      </c>
+      <c r="O9" t="n">
+        <v>0.4212854927252067</v>
+      </c>
+      <c r="P9" t="n">
+        <v>0.4236115578963774</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>0.4472135954999579</v>
+      </c>
+      <c r="R9" t="n">
+        <v>0.3704367657024817</v>
+      </c>
+      <c r="S9" t="n">
+        <v>0.3415515886228851</v>
+      </c>
+      <c r="T9" t="n">
+        <v>0.3768267838819982</v>
+      </c>
+      <c r="U9" t="n">
+        <v>0.3675741906306866</v>
+      </c>
+      <c r="V9" t="n">
+        <v>0.4472135954999579</v>
+      </c>
+      <c r="W9" t="n">
+        <v>0.4598925759210001</v>
+      </c>
+      <c r="X9" t="n">
+        <v>0.4140917151782204</v>
+      </c>
+      <c r="Y9" t="n">
+        <v>0.4558455495281818</v>
+      </c>
+      <c r="Z9" t="n">
+        <v>0.4569363138320738</v>
+      </c>
+      <c r="AA9" t="n">
+        <v>0.4472135954999579</v>
+      </c>
+      <c r="AB9" t="n">
+        <v>0.4870043257487428</v>
+      </c>
+      <c r="AC9" t="n">
+        <v>0.4431867587416085</v>
+      </c>
+      <c r="AD9" t="n">
+        <v>0.4910133034994928</v>
+      </c>
+      <c r="AE9" t="n">
+        <v>0.4814901592183074</v>
+      </c>
+      <c r="AF9" t="n">
+        <v>0.4472135954999579</v>
+      </c>
+      <c r="AG9" t="n">
+        <v>0.4470293253794135</v>
+      </c>
+      <c r="AH9" t="n">
+        <v>0.414395234732183</v>
+      </c>
+      <c r="AI9" t="n">
+        <v>0.4441932107907695</v>
+      </c>
+      <c r="AJ9" t="n">
+        <v>0.4448071973146608</v>
+      </c>
+      <c r="AK9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL9" t="n">
+        <v>0.1485767156532186</v>
+      </c>
+      <c r="AM9" t="n">
+        <v>0.1766592515118739</v>
+      </c>
+      <c r="AN9" t="n">
+        <v>0.1409833186875777</v>
+      </c>
+      <c r="AO9" t="n">
+        <v>0.1607189984478839</v>
+      </c>
+      <c r="AP9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ9" t="n">
+        <v>0.05025686602566577</v>
+      </c>
+      <c r="AR9" t="n">
+        <v>0.0868420746711223</v>
+      </c>
+      <c r="AS9" t="n">
+        <v>0.05746168108188222</v>
+      </c>
+      <c r="AT9" t="n">
+        <v>0.0760117042319861</v>
+      </c>
+      <c r="AU9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV9" t="n">
+        <v>0.04749116049392684</v>
+      </c>
+      <c r="AW9" t="n">
+        <v>0.07858330124326965</v>
+      </c>
+      <c r="AX9" t="n">
+        <v>0.06341618410332273</v>
+      </c>
+      <c r="AY9" t="n">
+        <v>0.06587518295912001</v>
+      </c>
+      <c r="AZ9" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA9" t="n">
+        <v>0.08247721154412875</v>
+      </c>
+      <c r="BB9" t="n">
+        <v>0.1100016128056689</v>
+      </c>
+      <c r="BC9" t="n">
+        <v>0.08440093287716685</v>
+      </c>
+      <c r="BD9" t="n">
+        <v>0.1003719994628212</v>
+      </c>
+      <c r="BE9" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF9" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG9" t="n">
+        <v>0.02051944134920436</v>
+      </c>
+      <c r="BH9" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI9" t="n">
+        <v>0.002687993818039751</v>
+      </c>
+      <c r="BJ9" t="inlineStr"/>
+      <c r="BK9" t="inlineStr"/>
+      <c r="BL9" t="inlineStr"/>
+      <c r="BM9" t="inlineStr"/>
+      <c r="BN9" t="inlineStr"/>
+      <c r="BO9" t="inlineStr"/>
+      <c r="BP9" t="inlineStr"/>
+      <c r="BQ9" t="inlineStr"/>
+      <c r="BR9" t="inlineStr"/>
+      <c r="BS9" t="inlineStr"/>
+      <c r="BT9" t="inlineStr"/>
+      <c r="BU9" t="inlineStr"/>
+      <c r="BV9" t="inlineStr"/>
+      <c r="BW9" t="inlineStr"/>
+      <c r="BX9" t="inlineStr"/>
+      <c r="BY9" t="inlineStr"/>
+      <c r="BZ9" t="inlineStr"/>
+      <c r="CA9" t="inlineStr"/>
+      <c r="CB9" t="inlineStr"/>
+      <c r="CC9" t="inlineStr"/>
+      <c r="CD9" t="inlineStr"/>
+      <c r="CE9" t="inlineStr"/>
+      <c r="CF9" t="inlineStr"/>
+      <c r="CG9" t="inlineStr"/>
+      <c r="CH9" t="inlineStr"/>
+      <c r="CI9" t="inlineStr"/>
+      <c r="CJ9" t="inlineStr"/>
+      <c r="CK9" t="inlineStr"/>
+      <c r="CL9" t="inlineStr"/>
+      <c r="CM9" t="inlineStr"/>
+      <c r="CN9" t="inlineStr"/>
+      <c r="CO9" t="inlineStr"/>
+      <c r="CP9" t="inlineStr"/>
+      <c r="CQ9" t="inlineStr"/>
+      <c r="CR9" t="inlineStr"/>
+      <c r="CS9" t="inlineStr"/>
+      <c r="CT9" t="inlineStr"/>
+      <c r="CU9" t="inlineStr"/>
+      <c r="CV9" t="inlineStr"/>
+      <c r="CW9" t="inlineStr"/>
+      <c r="CX9" t="inlineStr"/>
+      <c r="CY9" t="inlineStr"/>
+      <c r="CZ9" t="inlineStr"/>
+      <c r="DA9" t="inlineStr"/>
+      <c r="DB9" t="inlineStr"/>
+      <c r="DC9" t="inlineStr"/>
+      <c r="DD9" t="inlineStr"/>
+      <c r="DE9" t="inlineStr"/>
+      <c r="DF9" t="inlineStr"/>
+      <c r="DG9" t="inlineStr"/>
+      <c r="DH9" t="inlineStr"/>
+      <c r="DI9" t="inlineStr"/>
+      <c r="DJ9" t="inlineStr"/>
+      <c r="DK9" t="inlineStr"/>
+      <c r="DL9" t="inlineStr"/>
+      <c r="DM9" t="inlineStr"/>
+      <c r="DN9" t="inlineStr"/>
+      <c r="DO9" t="inlineStr"/>
+      <c r="DP9" t="inlineStr"/>
+      <c r="DQ9" t="inlineStr"/>
+      <c r="DR9" t="inlineStr"/>
+      <c r="DS9" t="inlineStr"/>
+      <c r="DT9" t="inlineStr"/>
+      <c r="DU9" t="inlineStr"/>
+      <c r="DV9" t="inlineStr"/>
+      <c r="DW9" t="inlineStr"/>
+      <c r="DX9" t="inlineStr"/>
+      <c r="DY9" t="inlineStr"/>
+      <c r="DZ9" t="inlineStr"/>
+      <c r="EA9" t="inlineStr"/>
+      <c r="EB9" t="inlineStr"/>
+      <c r="EC9" t="inlineStr"/>
+      <c r="ED9" t="inlineStr"/>
+      <c r="EE9" t="inlineStr"/>
+      <c r="EF9" t="inlineStr"/>
+      <c r="EG9" t="inlineStr"/>
+      <c r="EH9" t="inlineStr"/>
+      <c r="EI9" t="inlineStr"/>
+      <c r="EJ9" t="inlineStr"/>
+      <c r="EK9" t="inlineStr"/>
+      <c r="EL9" t="inlineStr"/>
+      <c r="EM9" t="inlineStr"/>
+      <c r="EN9" t="inlineStr"/>
+      <c r="EO9" t="inlineStr"/>
+      <c r="EP9" t="inlineStr"/>
+      <c r="EQ9" t="inlineStr"/>
+      <c r="ER9" t="inlineStr"/>
+      <c r="ES9" t="inlineStr"/>
+      <c r="ET9" t="inlineStr"/>
+      <c r="EU9" t="inlineStr"/>
+      <c r="EV9" t="inlineStr"/>
+      <c r="EW9" t="inlineStr"/>
+      <c r="EX9" t="inlineStr"/>
+      <c r="EY9" t="inlineStr"/>
+      <c r="EZ9" t="inlineStr"/>
+      <c r="FA9" t="inlineStr"/>
+      <c r="FB9" t="inlineStr"/>
+      <c r="FC9" t="inlineStr"/>
+      <c r="FD9" t="inlineStr"/>
+      <c r="FE9" t="inlineStr"/>
+      <c r="FF9" t="inlineStr"/>
+      <c r="FG9" t="inlineStr"/>
+      <c r="FH9" t="inlineStr"/>
+      <c r="FI9" t="inlineStr"/>
+      <c r="FJ9" t="inlineStr"/>
+      <c r="FK9" t="inlineStr"/>
+      <c r="FL9" t="inlineStr"/>
+      <c r="FM9" t="inlineStr"/>
+      <c r="FN9" t="inlineStr"/>
+      <c r="FO9" t="inlineStr"/>
+      <c r="FP9" t="inlineStr"/>
+      <c r="FQ9" t="inlineStr"/>
+      <c r="FR9" t="inlineStr"/>
+      <c r="FS9" t="inlineStr"/>
+      <c r="FT9" t="inlineStr"/>
+      <c r="FU9" t="inlineStr"/>
+      <c r="FV9" t="inlineStr"/>
+      <c r="FW9" t="inlineStr"/>
+      <c r="FX9" t="inlineStr"/>
+      <c r="FY9" t="inlineStr"/>
+      <c r="FZ9" t="inlineStr"/>
+      <c r="GA9" t="inlineStr"/>
+      <c r="GB9" t="inlineStr"/>
+      <c r="GC9" t="inlineStr"/>
+      <c r="GD9" t="inlineStr"/>
+      <c r="GE9" t="inlineStr"/>
+      <c r="GF9" t="inlineStr"/>
+      <c r="GG9" t="inlineStr"/>
+      <c r="GH9" t="inlineStr"/>
+      <c r="GI9" t="inlineStr"/>
+      <c r="GJ9" t="inlineStr"/>
+      <c r="GK9" t="inlineStr"/>
+      <c r="GL9" t="inlineStr"/>
+      <c r="GM9" t="inlineStr"/>
+      <c r="GN9" t="inlineStr"/>
+      <c r="GO9" t="inlineStr"/>
+      <c r="GP9" t="inlineStr"/>
+      <c r="GQ9" t="inlineStr"/>
+      <c r="GR9" t="inlineStr"/>
+      <c r="GS9" t="inlineStr"/>
+      <c r="GT9" t="inlineStr"/>
+      <c r="GU9" t="inlineStr"/>
+      <c r="GV9" t="inlineStr"/>
+      <c r="GW9" t="inlineStr"/>
+      <c r="GX9" t="inlineStr"/>
+      <c r="GY9" t="inlineStr"/>
+      <c r="GZ9" t="inlineStr"/>
+      <c r="HA9" t="inlineStr"/>
+      <c r="HB9" t="inlineStr"/>
+      <c r="HC9" t="inlineStr"/>
+      <c r="HD9" t="inlineStr"/>
+      <c r="HE9" t="inlineStr"/>
+      <c r="HF9" t="inlineStr"/>
+      <c r="HG9" t="inlineStr"/>
+      <c r="HH9" t="inlineStr"/>
+      <c r="HI9" t="inlineStr"/>
+      <c r="HJ9" t="inlineStr"/>
+      <c r="HK9" t="inlineStr"/>
+      <c r="HL9" t="inlineStr"/>
+      <c r="HM9" t="inlineStr"/>
+      <c r="HN9" t="inlineStr"/>
+      <c r="HO9" t="inlineStr"/>
+      <c r="HP9" t="inlineStr"/>
+      <c r="HQ9" t="inlineStr"/>
+      <c r="HR9" t="inlineStr"/>
+      <c r="HS9" t="inlineStr"/>
+      <c r="HT9" t="inlineStr"/>
+      <c r="HU9" t="inlineStr"/>
+      <c r="HV9" t="inlineStr"/>
+      <c r="HW9" t="inlineStr"/>
+      <c r="HX9" t="inlineStr"/>
+      <c r="HY9" t="inlineStr"/>
+      <c r="HZ9" t="inlineStr"/>
+      <c r="IA9" t="inlineStr"/>
+      <c r="IB9" t="inlineStr"/>
+      <c r="IC9" t="inlineStr"/>
+      <c r="ID9" t="inlineStr"/>
+      <c r="IE9" t="inlineStr"/>
+      <c r="IF9" t="inlineStr"/>
+      <c r="IG9" t="inlineStr"/>
+      <c r="IH9" t="inlineStr"/>
+      <c r="II9" t="inlineStr"/>
+      <c r="IJ9" t="inlineStr"/>
+      <c r="IK9" t="inlineStr"/>
+      <c r="IL9" t="inlineStr"/>
+      <c r="IM9" t="inlineStr"/>
+      <c r="IN9" t="inlineStr"/>
+      <c r="IO9" t="inlineStr"/>
+      <c r="IP9" t="inlineStr"/>
+      <c r="IQ9" t="inlineStr"/>
+      <c r="IR9" t="inlineStr"/>
+      <c r="IS9" t="inlineStr"/>
+      <c r="IT9" t="inlineStr"/>
+      <c r="IU9" t="inlineStr"/>
+      <c r="IV9" t="inlineStr"/>
+      <c r="IW9" t="inlineStr"/>
+      <c r="IX9" t="inlineStr"/>
+      <c r="IY9" t="inlineStr"/>
+      <c r="IZ9" t="inlineStr"/>
+      <c r="JA9" t="inlineStr"/>
+      <c r="JB9" t="inlineStr"/>
+      <c r="JC9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-04-15 20:41:32</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>10</v>
+      </c>
+      <c r="C10" t="n">
+        <v>100</v>
+      </c>
+      <c r="D10" t="n">
+        <v>50</v>
+      </c>
+      <c r="E10" t="n">
+        <v>50</v>
+      </c>
+      <c r="F10" t="n">
+        <v>5</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
+        <v>0.1838516269916657</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0.512665407645299</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0.1630754666328138</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0.3706923598207267</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0.4472135954999579</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0.5426102878355851</v>
+      </c>
+      <c r="N10" t="n">
+        <v>0.3338797321802806</v>
+      </c>
+      <c r="O10" t="n">
+        <v>0.5247927382940825</v>
+      </c>
+      <c r="P10" t="n">
+        <v>0.4717167956663637</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>0.4472135954999579</v>
+      </c>
+      <c r="R10" t="n">
+        <v>0.4765110931183587</v>
+      </c>
+      <c r="S10" t="n">
+        <v>0.2904214012501027</v>
+      </c>
+      <c r="T10" t="n">
+        <v>0.4642355707261704</v>
+      </c>
+      <c r="U10" t="n">
+        <v>0.4422579284161834</v>
+      </c>
+      <c r="V10" t="n">
+        <v>0.4472135954999579</v>
+      </c>
+      <c r="W10" t="n">
+        <v>0.4152108564637077</v>
+      </c>
+      <c r="X10" t="n">
+        <v>0.256968058618641</v>
+      </c>
+      <c r="Y10" t="n">
+        <v>0.4391582950457917</v>
+      </c>
+      <c r="Z10" t="n">
+        <v>0.4051626907151963</v>
+      </c>
+      <c r="AA10" t="n">
+        <v>0.4472135954999579</v>
+      </c>
+      <c r="AB10" t="n">
+        <v>0.3704450098461272</v>
+      </c>
+      <c r="AC10" t="n">
+        <v>0.2315601995760841</v>
+      </c>
+      <c r="AD10" t="n">
+        <v>0.3830621116547569</v>
+      </c>
+      <c r="AE10" t="n">
+        <v>0.378742683526372</v>
+      </c>
+      <c r="AF10" t="n">
+        <v>0.4472135954999579</v>
+      </c>
+      <c r="AG10" t="n">
+        <v>0.3934995929722896</v>
+      </c>
+      <c r="AH10" t="n">
+        <v>0.2517793474874719</v>
+      </c>
+      <c r="AI10" t="n">
+        <v>0.3950867043555272</v>
+      </c>
+      <c r="AJ10" t="n">
+        <v>0.380817398510826</v>
+      </c>
+      <c r="AK10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL10" t="n">
+        <v>3.402980168117167e-05</v>
+      </c>
+      <c r="AM10" t="n">
+        <v>0.03213758516822962</v>
+      </c>
+      <c r="AN10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO10" t="n">
+        <v>0.03298242155452278</v>
+      </c>
+      <c r="AP10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR10" t="n">
+        <v>0.01269718614916328</v>
+      </c>
+      <c r="AS10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT10" t="n">
+        <v>0.0106882844325721</v>
+      </c>
+      <c r="AU10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW10" t="n">
+        <v>0.04411102269612127</v>
+      </c>
+      <c r="AX10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY10" t="n">
+        <v>0.04226166828901452</v>
+      </c>
+      <c r="AZ10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB10" t="n">
+        <v>0.03638821067383498</v>
+      </c>
+      <c r="BC10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD10" t="n">
+        <v>0.01681901334844079</v>
+      </c>
+      <c r="BE10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG10" t="n">
+        <v>0.05879325592237104</v>
+      </c>
+      <c r="BH10" t="n">
+        <v>0.0008523556492664462</v>
+      </c>
+      <c r="BI10" t="n">
+        <v>0.06162362132781011</v>
+      </c>
+      <c r="BJ10" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="BK10" t="n">
+        <v>0.9498778778778779</v>
+      </c>
+      <c r="BL10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN10" t="n">
+        <v>0.00174627505960817</v>
+      </c>
+      <c r="BO10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP10" t="n">
+        <v>-0.02880239405345075</v>
+      </c>
+      <c r="BQ10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BR10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BS10" t="n">
+        <v>0.01932549567286986</v>
+      </c>
+      <c r="BT10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU10" t="n">
+        <v>-0.01653855485122683</v>
+      </c>
+      <c r="BV10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW10" t="n">
+        <v>4.222484932484335e-05</v>
+      </c>
+      <c r="BX10" t="n">
+        <v>0.03075204775195141</v>
+      </c>
+      <c r="BY10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BZ10" t="n">
+        <v>0.01412941753310348</v>
+      </c>
+      <c r="CA10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CB10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CC10" t="n">
+        <v>0.03871919829033913</v>
+      </c>
+      <c r="CD10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CE10" t="n">
+        <v>0.01855925052400355</v>
+      </c>
+      <c r="CF10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CG10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CH10" t="n">
+        <v>0.03835895997683601</v>
+      </c>
+      <c r="CI10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CJ10" t="n">
+        <v>0.01002283617893552</v>
+      </c>
+      <c r="CK10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL10" t="n">
+        <v>0.01447829428012932</v>
+      </c>
+      <c r="CM10" t="n">
+        <v>0.08219233943161922</v>
+      </c>
+      <c r="CN10" t="n">
+        <v>0.004724393950496597</v>
+      </c>
+      <c r="CO10" t="n">
+        <v>0.06141832673640824</v>
+      </c>
+      <c r="CP10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR10" t="n">
+        <v>0.01097820889160808</v>
+      </c>
+      <c r="CS10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CT10" t="n">
+        <v>-0.03690601230919455</v>
+      </c>
+      <c r="CU10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CV10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW10" t="n">
+        <v>0.02114881452869118</v>
+      </c>
+      <c r="CX10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CY10" t="n">
+        <v>-0.002666310391341191</v>
+      </c>
+      <c r="CZ10" t="n">
+        <v>0</v>
+      </c>
+      <c r="DA10" t="n">
+        <v>1.466399810915956e-05</v>
+      </c>
+      <c r="DB10" t="n">
+        <v>0.04327880803388323</v>
+      </c>
+      <c r="DC10" t="n">
+        <v>0</v>
+      </c>
+      <c r="DD10" t="n">
+        <v>0.0312109021986321</v>
+      </c>
+      <c r="DE10" t="n">
+        <v>0</v>
+      </c>
+      <c r="DF10" t="n">
+        <v>2.566447998067225e-06</v>
+      </c>
+      <c r="DG10" t="n">
+        <v>0.03990042265394066</v>
+      </c>
+      <c r="DH10" t="n">
+        <v>0</v>
+      </c>
+      <c r="DI10" t="n">
+        <v>0.0002769818918783444</v>
+      </c>
+      <c r="DJ10" t="n">
+        <v>0</v>
+      </c>
+      <c r="DK10" t="n">
+        <v>0.002407430485358878</v>
+      </c>
+      <c r="DL10" t="n">
+        <v>0.06336310452480753</v>
+      </c>
+      <c r="DM10" t="n">
+        <v>0.002445414673552631</v>
+      </c>
+      <c r="DN10" t="n">
+        <v>0.07916985799375562</v>
+      </c>
+      <c r="DO10" t="n">
+        <v>0</v>
+      </c>
+      <c r="DP10" t="n">
+        <v>2.000421337456229e-05</v>
+      </c>
+      <c r="DQ10" t="n">
+        <v>0.006833387500124431</v>
+      </c>
+      <c r="DR10" t="n">
+        <v>0</v>
+      </c>
+      <c r="DS10" t="n">
+        <v>0.002486171611522787</v>
+      </c>
+      <c r="DT10" t="n">
+        <v>0</v>
+      </c>
+      <c r="DU10" t="n">
+        <v>4.590091240107541e-06</v>
+      </c>
+      <c r="DV10" t="n">
+        <v>0.0135123323342331</v>
+      </c>
+      <c r="DW10" t="n">
+        <v>0</v>
+      </c>
+      <c r="DX10" t="n">
+        <v>0.00807596186700189</v>
+      </c>
+      <c r="DY10" t="n">
+        <v>0</v>
+      </c>
+      <c r="DZ10" t="n">
+        <v>0</v>
+      </c>
+      <c r="EA10" t="n">
+        <v>0.02924195065874801</v>
+      </c>
+      <c r="EB10" t="n">
+        <v>0</v>
+      </c>
+      <c r="EC10" t="n">
+        <v>0.01901106571408978</v>
+      </c>
+      <c r="ED10" t="n">
+        <v>0</v>
+      </c>
+      <c r="EE10" t="n">
+        <v>0.009427882058312288</v>
+      </c>
+      <c r="EF10" t="n">
+        <v>0.08309402595095965</v>
+      </c>
+      <c r="EG10" t="n">
+        <v>0</v>
+      </c>
+      <c r="EH10" t="n">
+        <v>0.07242200518991034</v>
+      </c>
+      <c r="EI10" t="n">
+        <v>0</v>
+      </c>
+      <c r="EJ10" t="n">
+        <v>0</v>
+      </c>
+      <c r="EK10" t="n">
+        <v>-0.02400918976652706</v>
+      </c>
+      <c r="EL10" t="n">
+        <v>0</v>
+      </c>
+      <c r="EM10" t="n">
+        <v>-0.07213495670444392</v>
+      </c>
+      <c r="EN10" t="n">
+        <v>0</v>
+      </c>
+      <c r="EO10" t="n">
+        <v>2.109216419940168e-05</v>
+      </c>
+      <c r="EP10" t="n">
+        <v>0.01135569381840972</v>
+      </c>
+      <c r="EQ10" t="n">
+        <v>0</v>
+      </c>
+      <c r="ER10" t="n">
+        <v>-0.02509527946170018</v>
+      </c>
+      <c r="ES10" t="n">
+        <v>0</v>
+      </c>
+      <c r="ET10" t="n">
+        <v>9.85218990472901e-06</v>
+      </c>
+      <c r="EU10" t="n">
+        <v>0.04577119432450395</v>
+      </c>
+      <c r="EV10" t="n">
+        <v>0</v>
+      </c>
+      <c r="EW10" t="n">
+        <v>0.04235868152814665</v>
+      </c>
+      <c r="EX10" t="n">
+        <v>0</v>
+      </c>
+      <c r="EY10" t="n">
+        <v>0</v>
+      </c>
+      <c r="EZ10" t="n">
+        <v>-0.0002097365405444654</v>
+      </c>
+      <c r="FA10" t="n">
+        <v>0</v>
+      </c>
+      <c r="FB10" t="n">
+        <v>-0.06118441210219847</v>
+      </c>
+      <c r="FC10" t="n">
+        <v>0</v>
+      </c>
+      <c r="FD10" t="n">
+        <v>0</v>
+      </c>
+      <c r="FE10" t="n">
+        <v>0.04716357064125912</v>
+      </c>
+      <c r="FF10" t="n">
+        <v>0</v>
+      </c>
+      <c r="FG10" t="n">
+        <v>0.04185667135170823</v>
+      </c>
+      <c r="FH10" t="n">
+        <v>0</v>
+      </c>
+      <c r="FI10" t="n">
+        <v>0</v>
+      </c>
+      <c r="FJ10" t="n">
+        <v>0.06681722639409794</v>
+      </c>
+      <c r="FK10" t="n">
+        <v>0</v>
+      </c>
+      <c r="FL10" t="n">
+        <v>0.03999737585137323</v>
+      </c>
+      <c r="FM10" t="n">
+        <v>0</v>
+      </c>
+      <c r="FN10" t="n">
+        <v>5.878311971236692e-06</v>
+      </c>
+      <c r="FO10" t="n">
+        <v>0.03841304717534481</v>
+      </c>
+      <c r="FP10" t="n">
+        <v>0</v>
+      </c>
+      <c r="FQ10" t="n">
+        <v>0.02155994385208829</v>
+      </c>
+      <c r="FR10" t="n">
+        <v>0</v>
+      </c>
+      <c r="FS10" t="n">
+        <v>0.02830456116024311</v>
+      </c>
+      <c r="FT10" t="n">
+        <v>0.08972065342534727</v>
+      </c>
+      <c r="FU10" t="n">
+        <v>0.02032707530120384</v>
+      </c>
+      <c r="FV10" t="n">
+        <v>0.09265000316290524</v>
+      </c>
+      <c r="FW10" t="n">
+        <v>0</v>
+      </c>
+      <c r="FX10" t="n">
+        <v>1.130904622296478e-05</v>
+      </c>
+      <c r="FY10" t="n">
+        <v>0.02878995476973052</v>
+      </c>
+      <c r="FZ10" t="n">
+        <v>0</v>
+      </c>
+      <c r="GA10" t="n">
+        <v>0.003462919326619284</v>
+      </c>
+      <c r="GB10" t="n">
+        <v>0</v>
+      </c>
+      <c r="GC10" t="n">
+        <v>0</v>
+      </c>
+      <c r="GD10" t="n">
+        <v>0.005205481851621524</v>
+      </c>
+      <c r="GE10" t="n">
+        <v>0</v>
+      </c>
+      <c r="GF10" t="n">
+        <v>-0.03156361145421006</v>
+      </c>
+      <c r="GG10" t="n">
+        <v>0</v>
+      </c>
+      <c r="GH10" t="n">
+        <v>0.09322997473552375</v>
+      </c>
+      <c r="GI10" t="n">
+        <v>0.09924442858974353</v>
+      </c>
+      <c r="GJ10" t="n">
+        <v>0.1020109457116977</v>
+      </c>
+      <c r="GK10" t="n">
+        <v>0.1580575732770333</v>
+      </c>
+      <c r="GL10" t="n">
+        <v>0</v>
+      </c>
+      <c r="GM10" t="n">
+        <v>0.003546019636902043</v>
+      </c>
+      <c r="GN10" t="n">
+        <v>0.07955937313271948</v>
+      </c>
+      <c r="GO10" t="n">
+        <v>0</v>
+      </c>
+      <c r="GP10" t="n">
+        <v>0.05762591213102712</v>
+      </c>
+      <c r="GQ10" t="n">
+        <v>0</v>
+      </c>
+      <c r="GR10" t="n">
+        <v>9.810753245881939e-06</v>
+      </c>
+      <c r="GS10" t="n">
+        <v>0.03257200300310992</v>
+      </c>
+      <c r="GT10" t="n">
+        <v>0</v>
+      </c>
+      <c r="GU10" t="n">
+        <v>-0.005032452471484753</v>
+      </c>
+      <c r="GV10" t="n">
+        <v>0</v>
+      </c>
+      <c r="GW10" t="n">
+        <v>0</v>
+      </c>
+      <c r="GX10" t="n">
+        <v>0.009624252295213968</v>
+      </c>
+      <c r="GY10" t="n">
+        <v>0</v>
+      </c>
+      <c r="GZ10" t="n">
+        <v>-0.004916250253375393</v>
+      </c>
+      <c r="HA10" t="n">
+        <v>0</v>
+      </c>
+      <c r="HB10" t="n">
+        <v>1.751041721737505e-05</v>
+      </c>
+      <c r="HC10" t="n">
+        <v>0.03352095517755536</v>
+      </c>
+      <c r="HD10" t="n">
+        <v>0</v>
+      </c>
+      <c r="HE10" t="n">
+        <v>0.01844851227270021</v>
+      </c>
+      <c r="HF10" t="n">
+        <v>0</v>
+      </c>
+      <c r="HG10" t="n">
+        <v>0.03623727805208501</v>
+      </c>
+      <c r="HH10" t="n">
+        <v>0.08212761042941319</v>
+      </c>
+      <c r="HI10" t="n">
+        <v>0.02493666992486772</v>
+      </c>
+      <c r="HJ10" t="n">
+        <v>0.09798305622363936</v>
+      </c>
+      <c r="HK10" t="n">
+        <v>0</v>
+      </c>
+      <c r="HL10" t="n">
+        <v>0</v>
+      </c>
+      <c r="HM10" t="n">
+        <v>0.01238561433255004</v>
+      </c>
+      <c r="HN10" t="n">
+        <v>0</v>
+      </c>
+      <c r="HO10" t="n">
+        <v>0.009751271096852573</v>
+      </c>
+      <c r="HP10" t="n">
+        <v>0</v>
+      </c>
+      <c r="HQ10" t="n">
+        <v>3.063636560625645e-06</v>
+      </c>
+      <c r="HR10" t="n">
+        <v>0.0001049190459050775</v>
+      </c>
+      <c r="HS10" t="n">
+        <v>0</v>
+      </c>
+      <c r="HT10" t="n">
+        <v>-0.03837435582968256</v>
+      </c>
+      <c r="HU10" t="n">
+        <v>0</v>
+      </c>
+      <c r="HV10" t="n">
+        <v>0.02464531518298731</v>
+      </c>
+      <c r="HW10" t="n">
+        <v>0.08711306121510076</v>
+      </c>
+      <c r="HX10" t="n">
+        <v>0</v>
+      </c>
+      <c r="HY10" t="n">
+        <v>0.08934917130341594</v>
+      </c>
+      <c r="HZ10" t="n">
+        <v>0</v>
+      </c>
+      <c r="IA10" t="n">
+        <v>0</v>
+      </c>
+      <c r="IB10" t="n">
+        <v>-0.02622461161365992</v>
+      </c>
+      <c r="IC10" t="n">
+        <v>0</v>
+      </c>
+      <c r="ID10" t="n">
+        <v>-0.05451751306570535</v>
+      </c>
+      <c r="IE10" t="n">
+        <v>0</v>
+      </c>
+      <c r="IF10" t="n">
+        <v>2.84317544800809e-06</v>
+      </c>
+      <c r="IG10" t="n">
+        <v>0.01525429230278179</v>
+      </c>
+      <c r="IH10" t="n">
+        <v>0</v>
+      </c>
+      <c r="II10" t="n">
+        <v>-0.01597344351631224</v>
+      </c>
+      <c r="IJ10" t="n">
+        <v>0</v>
+      </c>
+      <c r="IK10" t="n">
+        <v>0.002193485659900803</v>
+      </c>
+      <c r="IL10" t="n">
+        <v>0.06101763468567134</v>
+      </c>
+      <c r="IM10" t="n">
+        <v>0.01796713692626386</v>
+      </c>
+      <c r="IN10" t="n">
+        <v>0.07698585834338659</v>
+      </c>
+      <c r="IO10" t="n">
+        <v>0</v>
+      </c>
+      <c r="IP10" t="n">
+        <v>0.04800586498262757</v>
+      </c>
+      <c r="IQ10" t="n">
+        <v>0.08737200100479445</v>
+      </c>
+      <c r="IR10" t="n">
+        <v>0.03993392344940688</v>
+      </c>
+      <c r="IS10" t="n">
+        <v>0.1140274349804736</v>
+      </c>
+      <c r="IT10" t="n">
+        <v>0</v>
+      </c>
+      <c r="IU10" t="n">
+        <v>0</v>
+      </c>
+      <c r="IV10" t="n">
+        <v>0.05464298669358475</v>
+      </c>
+      <c r="IW10" t="n">
+        <v>0</v>
+      </c>
+      <c r="IX10" t="n">
+        <v>0.04320282427780254</v>
+      </c>
+      <c r="IY10" t="n">
+        <v>0</v>
+      </c>
+      <c r="IZ10" t="n">
+        <v>0</v>
+      </c>
+      <c r="JA10" t="n">
+        <v>0.03768344605585518</v>
+      </c>
+      <c r="JB10" t="n">
+        <v>0</v>
+      </c>
+      <c r="JC10" t="n">
+        <v>0.04897292210852509</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
some nasty bugs found
</commit_message>
<xml_diff>
--- a/ranking/results.xlsx
+++ b/ranking/results.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:JC69"/>
+  <dimension ref="A1:JD72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1744,6 +1744,11 @@
           <t>theta_49_dgd</t>
         </is>
       </c>
+      <c r="JD1" s="1" t="inlineStr">
+        <is>
+          <t>W_inner</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2539,6 +2544,7 @@
       <c r="JC2" t="n">
         <v>0.09899675505170645</v>
       </c>
+      <c r="JD2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3028,6 +3034,7 @@
       <c r="JA3" t="inlineStr"/>
       <c r="JB3" t="inlineStr"/>
       <c r="JC3" t="inlineStr"/>
+      <c r="JD3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3517,6 +3524,7 @@
       <c r="JA4" t="inlineStr"/>
       <c r="JB4" t="inlineStr"/>
       <c r="JC4" t="inlineStr"/>
+      <c r="JD4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -4006,6 +4014,7 @@
       <c r="JA5" t="inlineStr"/>
       <c r="JB5" t="inlineStr"/>
       <c r="JC5" t="inlineStr"/>
+      <c r="JD5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -4495,6 +4504,7 @@
       <c r="JA6" t="inlineStr"/>
       <c r="JB6" t="inlineStr"/>
       <c r="JC6" t="inlineStr"/>
+      <c r="JD6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -4984,6 +4994,7 @@
       <c r="JA7" t="inlineStr"/>
       <c r="JB7" t="inlineStr"/>
       <c r="JC7" t="inlineStr"/>
+      <c r="JD7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -5473,6 +5484,7 @@
       <c r="JA8" t="inlineStr"/>
       <c r="JB8" t="inlineStr"/>
       <c r="JC8" t="inlineStr"/>
+      <c r="JD8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -5962,6 +5974,7 @@
       <c r="JA9" t="inlineStr"/>
       <c r="JB9" t="inlineStr"/>
       <c r="JC9" t="inlineStr"/>
+      <c r="JD9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -6451,6 +6464,7 @@
       <c r="JA10" t="inlineStr"/>
       <c r="JB10" t="inlineStr"/>
       <c r="JC10" t="inlineStr"/>
+      <c r="JD10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -6940,6 +6954,7 @@
       <c r="JA11" t="inlineStr"/>
       <c r="JB11" t="inlineStr"/>
       <c r="JC11" t="inlineStr"/>
+      <c r="JD11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -7429,6 +7444,7 @@
       <c r="JA12" t="inlineStr"/>
       <c r="JB12" t="inlineStr"/>
       <c r="JC12" t="inlineStr"/>
+      <c r="JD12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -7918,6 +7934,7 @@
       <c r="JA13" t="inlineStr"/>
       <c r="JB13" t="inlineStr"/>
       <c r="JC13" t="inlineStr"/>
+      <c r="JD13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -8407,6 +8424,7 @@
       <c r="JA14" t="inlineStr"/>
       <c r="JB14" t="inlineStr"/>
       <c r="JC14" t="inlineStr"/>
+      <c r="JD14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -8896,6 +8914,7 @@
       <c r="JA15" t="inlineStr"/>
       <c r="JB15" t="inlineStr"/>
       <c r="JC15" t="inlineStr"/>
+      <c r="JD15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -9385,6 +9404,7 @@
       <c r="JA16" t="inlineStr"/>
       <c r="JB16" t="inlineStr"/>
       <c r="JC16" t="inlineStr"/>
+      <c r="JD16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -9874,6 +9894,7 @@
       <c r="JA17" t="inlineStr"/>
       <c r="JB17" t="inlineStr"/>
       <c r="JC17" t="inlineStr"/>
+      <c r="JD17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -10363,6 +10384,7 @@
       <c r="JA18" t="inlineStr"/>
       <c r="JB18" t="inlineStr"/>
       <c r="JC18" t="inlineStr"/>
+      <c r="JD18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -10852,6 +10874,7 @@
       <c r="JA19" t="inlineStr"/>
       <c r="JB19" t="inlineStr"/>
       <c r="JC19" t="inlineStr"/>
+      <c r="JD19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -11341,6 +11364,7 @@
       <c r="JA20" t="inlineStr"/>
       <c r="JB20" t="inlineStr"/>
       <c r="JC20" t="inlineStr"/>
+      <c r="JD20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -11830,6 +11854,7 @@
       <c r="JA21" t="inlineStr"/>
       <c r="JB21" t="inlineStr"/>
       <c r="JC21" t="inlineStr"/>
+      <c r="JD21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -12319,6 +12344,7 @@
       <c r="JA22" t="inlineStr"/>
       <c r="JB22" t="inlineStr"/>
       <c r="JC22" t="inlineStr"/>
+      <c r="JD22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -12808,6 +12834,7 @@
       <c r="JA23" t="inlineStr"/>
       <c r="JB23" t="inlineStr"/>
       <c r="JC23" t="inlineStr"/>
+      <c r="JD23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -13297,6 +13324,7 @@
       <c r="JA24" t="inlineStr"/>
       <c r="JB24" t="inlineStr"/>
       <c r="JC24" t="inlineStr"/>
+      <c r="JD24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -13786,6 +13814,7 @@
       <c r="JA25" t="inlineStr"/>
       <c r="JB25" t="inlineStr"/>
       <c r="JC25" t="inlineStr"/>
+      <c r="JD25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -14275,6 +14304,7 @@
       <c r="JA26" t="inlineStr"/>
       <c r="JB26" t="inlineStr"/>
       <c r="JC26" t="inlineStr"/>
+      <c r="JD26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -14764,6 +14794,7 @@
       <c r="JA27" t="inlineStr"/>
       <c r="JB27" t="inlineStr"/>
       <c r="JC27" t="inlineStr"/>
+      <c r="JD27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -15253,6 +15284,7 @@
       <c r="JA28" t="inlineStr"/>
       <c r="JB28" t="inlineStr"/>
       <c r="JC28" t="inlineStr"/>
+      <c r="JD28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -15742,6 +15774,7 @@
       <c r="JA29" t="inlineStr"/>
       <c r="JB29" t="inlineStr"/>
       <c r="JC29" t="inlineStr"/>
+      <c r="JD29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -16231,6 +16264,7 @@
       <c r="JA30" t="inlineStr"/>
       <c r="JB30" t="inlineStr"/>
       <c r="JC30" t="inlineStr"/>
+      <c r="JD30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -16720,6 +16754,7 @@
       <c r="JA31" t="inlineStr"/>
       <c r="JB31" t="inlineStr"/>
       <c r="JC31" t="inlineStr"/>
+      <c r="JD31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -17209,6 +17244,7 @@
       <c r="JA32" t="inlineStr"/>
       <c r="JB32" t="inlineStr"/>
       <c r="JC32" t="inlineStr"/>
+      <c r="JD32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -17698,6 +17734,7 @@
       <c r="JA33" t="inlineStr"/>
       <c r="JB33" t="inlineStr"/>
       <c r="JC33" t="inlineStr"/>
+      <c r="JD33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -18187,6 +18224,7 @@
       <c r="JA34" t="inlineStr"/>
       <c r="JB34" t="inlineStr"/>
       <c r="JC34" t="inlineStr"/>
+      <c r="JD34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -18676,6 +18714,7 @@
       <c r="JA35" t="inlineStr"/>
       <c r="JB35" t="inlineStr"/>
       <c r="JC35" t="inlineStr"/>
+      <c r="JD35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -19165,6 +19204,7 @@
       <c r="JA36" t="inlineStr"/>
       <c r="JB36" t="inlineStr"/>
       <c r="JC36" t="inlineStr"/>
+      <c r="JD36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -19654,6 +19694,7 @@
       <c r="JA37" t="inlineStr"/>
       <c r="JB37" t="inlineStr"/>
       <c r="JC37" t="inlineStr"/>
+      <c r="JD37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -20143,6 +20184,7 @@
       <c r="JA38" t="inlineStr"/>
       <c r="JB38" t="inlineStr"/>
       <c r="JC38" t="inlineStr"/>
+      <c r="JD38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -20632,6 +20674,7 @@
       <c r="JA39" t="inlineStr"/>
       <c r="JB39" t="inlineStr"/>
       <c r="JC39" t="inlineStr"/>
+      <c r="JD39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -21121,6 +21164,7 @@
       <c r="JA40" t="inlineStr"/>
       <c r="JB40" t="inlineStr"/>
       <c r="JC40" t="inlineStr"/>
+      <c r="JD40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -21916,6 +21960,7 @@
       <c r="JC41" t="n">
         <v>0</v>
       </c>
+      <c r="JD41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -22711,6 +22756,7 @@
       <c r="JC42" t="n">
         <v>1.521290203721152e-05</v>
       </c>
+      <c r="JD42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -23200,6 +23246,7 @@
       <c r="JA43" t="inlineStr"/>
       <c r="JB43" t="inlineStr"/>
       <c r="JC43" t="inlineStr"/>
+      <c r="JD43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -23689,6 +23736,7 @@
       <c r="JA44" t="inlineStr"/>
       <c r="JB44" t="inlineStr"/>
       <c r="JC44" t="inlineStr"/>
+      <c r="JD44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -24178,6 +24226,7 @@
       <c r="JA45" t="inlineStr"/>
       <c r="JB45" t="inlineStr"/>
       <c r="JC45" t="inlineStr"/>
+      <c r="JD45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -24667,6 +24716,7 @@
       <c r="JA46" t="inlineStr"/>
       <c r="JB46" t="inlineStr"/>
       <c r="JC46" t="inlineStr"/>
+      <c r="JD46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -25156,6 +25206,7 @@
       <c r="JA47" t="inlineStr"/>
       <c r="JB47" t="inlineStr"/>
       <c r="JC47" t="inlineStr"/>
+      <c r="JD47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -25645,6 +25696,7 @@
       <c r="JA48" t="inlineStr"/>
       <c r="JB48" t="inlineStr"/>
       <c r="JC48" t="inlineStr"/>
+      <c r="JD48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -26134,6 +26186,7 @@
       <c r="JA49" t="inlineStr"/>
       <c r="JB49" t="inlineStr"/>
       <c r="JC49" t="inlineStr"/>
+      <c r="JD49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -26623,6 +26676,7 @@
       <c r="JA50" t="inlineStr"/>
       <c r="JB50" t="inlineStr"/>
       <c r="JC50" t="inlineStr"/>
+      <c r="JD50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -27112,6 +27166,7 @@
       <c r="JA51" t="inlineStr"/>
       <c r="JB51" t="inlineStr"/>
       <c r="JC51" t="inlineStr"/>
+      <c r="JD51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -27601,6 +27656,7 @@
       <c r="JA52" t="inlineStr"/>
       <c r="JB52" t="inlineStr"/>
       <c r="JC52" t="inlineStr"/>
+      <c r="JD52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -28090,6 +28146,7 @@
       <c r="JA53" t="inlineStr"/>
       <c r="JB53" t="inlineStr"/>
       <c r="JC53" t="inlineStr"/>
+      <c r="JD53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -28579,6 +28636,7 @@
       <c r="JA54" t="inlineStr"/>
       <c r="JB54" t="inlineStr"/>
       <c r="JC54" t="inlineStr"/>
+      <c r="JD54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -29068,6 +29126,7 @@
       <c r="JA55" t="inlineStr"/>
       <c r="JB55" t="inlineStr"/>
       <c r="JC55" t="inlineStr"/>
+      <c r="JD55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -29557,6 +29616,7 @@
       <c r="JA56" t="inlineStr"/>
       <c r="JB56" t="inlineStr"/>
       <c r="JC56" t="inlineStr"/>
+      <c r="JD56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -30046,6 +30106,7 @@
       <c r="JA57" t="inlineStr"/>
       <c r="JB57" t="inlineStr"/>
       <c r="JC57" t="inlineStr"/>
+      <c r="JD57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -30535,6 +30596,7 @@
       <c r="JA58" t="inlineStr"/>
       <c r="JB58" t="inlineStr"/>
       <c r="JC58" t="inlineStr"/>
+      <c r="JD58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -31024,6 +31086,7 @@
       <c r="JA59" t="inlineStr"/>
       <c r="JB59" t="inlineStr"/>
       <c r="JC59" t="inlineStr"/>
+      <c r="JD59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -31513,6 +31576,7 @@
       <c r="JA60" t="inlineStr"/>
       <c r="JB60" t="inlineStr"/>
       <c r="JC60" t="inlineStr"/>
+      <c r="JD60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -32002,6 +32066,7 @@
       <c r="JA61" t="inlineStr"/>
       <c r="JB61" t="inlineStr"/>
       <c r="JC61" t="inlineStr"/>
+      <c r="JD61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -32491,6 +32556,7 @@
       <c r="JA62" t="inlineStr"/>
       <c r="JB62" t="inlineStr"/>
       <c r="JC62" t="inlineStr"/>
+      <c r="JD62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -32980,6 +33046,7 @@
       <c r="JA63" t="inlineStr"/>
       <c r="JB63" t="inlineStr"/>
       <c r="JC63" t="inlineStr"/>
+      <c r="JD63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -33469,6 +33536,7 @@
       <c r="JA64" t="inlineStr"/>
       <c r="JB64" t="inlineStr"/>
       <c r="JC64" t="inlineStr"/>
+      <c r="JD64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -33958,6 +34026,7 @@
       <c r="JA65" t="inlineStr"/>
       <c r="JB65" t="inlineStr"/>
       <c r="JC65" t="inlineStr"/>
+      <c r="JD65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -34447,6 +34516,7 @@
       <c r="JA66" t="inlineStr"/>
       <c r="JB66" t="inlineStr"/>
       <c r="JC66" t="inlineStr"/>
+      <c r="JD66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -35242,6 +35312,7 @@
       <c r="JC67" t="n">
         <v>0.1201190150947564</v>
       </c>
+      <c r="JD67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -36037,6 +36108,7 @@
       <c r="JC68" t="n">
         <v>0.01666591981202987</v>
       </c>
+      <c r="JD68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -36212,7 +36284,7 @@
         <v>0.003724115605215337</v>
       </c>
       <c r="BE69" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="BF69" t="n">
         <v>-6.451094961079803e-05</v>
@@ -36236,7 +36308,7 @@
         <v>0</v>
       </c>
       <c r="BM69" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="BN69" t="n">
         <v>0.09617491420839436</v>
@@ -36251,7 +36323,7 @@
         <v>0</v>
       </c>
       <c r="BR69" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="BS69" t="n">
         <v>0.02178726416297033</v>
@@ -36266,7 +36338,7 @@
         <v>0</v>
       </c>
       <c r="BW69" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="BX69" t="n">
         <v>0.1092321448721939</v>
@@ -36281,7 +36353,7 @@
         <v>0</v>
       </c>
       <c r="CB69" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="CC69" t="n">
         <v>0.03145742493396329</v>
@@ -36296,7 +36368,7 @@
         <v>0</v>
       </c>
       <c r="CG69" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="CH69" t="n">
         <v>0.04800172339669577</v>
@@ -36311,7 +36383,7 @@
         <v>0</v>
       </c>
       <c r="CL69" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="CM69" t="n">
         <v>0.06772401197518638</v>
@@ -36371,13 +36443,13 @@
         <v>0</v>
       </c>
       <c r="DF69" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="DG69" t="n">
         <v>0.05939931194710104</v>
       </c>
       <c r="DH69" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="DI69" t="n">
         <v>1.226238473389266e-05</v>
@@ -36386,13 +36458,13 @@
         <v>0</v>
       </c>
       <c r="DK69" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="DL69" t="n">
         <v>0.008143156435312434</v>
       </c>
       <c r="DM69" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="DN69" t="n">
         <v>3.961425224824349e-06</v>
@@ -36416,13 +36488,13 @@
         <v>0</v>
       </c>
       <c r="DU69" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="DV69" t="n">
         <v>0.06738589146081003</v>
       </c>
       <c r="DW69" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="DX69" t="n">
         <v>-1.464848124137013e-05</v>
@@ -36437,7 +36509,7 @@
         <v>0.04867778281533248</v>
       </c>
       <c r="EB69" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="EC69" t="n">
         <v>-1.721245648697206e-05</v>
@@ -36446,7 +36518,7 @@
         <v>0</v>
       </c>
       <c r="EE69" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="EF69" t="n">
         <v>0.01226679541426947</v>
@@ -36461,7 +36533,7 @@
         <v>0</v>
       </c>
       <c r="EJ69" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="EK69" t="n">
         <v>-0.004253397733579068</v>
@@ -36482,7 +36554,7 @@
         <v>-0.0214507982942831</v>
       </c>
       <c r="EQ69" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="ER69" t="n">
         <v>-4.275784188696047e-05</v>
@@ -36491,13 +36563,13 @@
         <v>0</v>
       </c>
       <c r="ET69" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="EU69" t="n">
         <v>0.01464063127144998</v>
       </c>
       <c r="EV69" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="EW69" t="n">
         <v>-8.28241280239517e-06</v>
@@ -36506,13 +36578,13 @@
         <v>0</v>
       </c>
       <c r="EY69" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="EZ69" t="n">
         <v>-0.0606187468156335</v>
       </c>
       <c r="FA69" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="FB69" t="n">
         <v>-6.668065581172057e-05</v>
@@ -36521,7 +36593,7 @@
         <v>0</v>
       </c>
       <c r="FD69" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="FE69" t="n">
         <v>0.04289344924151425</v>
@@ -36536,13 +36608,13 @@
         <v>0</v>
       </c>
       <c r="FI69" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="FJ69" t="n">
         <v>-0.1289927253317418</v>
       </c>
       <c r="FK69" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="FL69" t="n">
         <v>-0.06763325675082377</v>
@@ -36551,13 +36623,13 @@
         <v>0</v>
       </c>
       <c r="FN69" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="FO69" t="n">
         <v>-0.01463331012582409</v>
       </c>
       <c r="FP69" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="FQ69" t="n">
         <v>-6.878839833613235e-05</v>
@@ -36566,13 +36638,13 @@
         <v>0</v>
       </c>
       <c r="FS69" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="FT69" t="n">
         <v>0.04123041033009264</v>
       </c>
       <c r="FU69" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="FV69" t="n">
         <v>-2.757026067083453e-05</v>
@@ -36581,7 +36653,7 @@
         <v>0</v>
       </c>
       <c r="FX69" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="FY69" t="n">
         <v>0.05486375645114731</v>
@@ -36602,7 +36674,7 @@
         <v>0.005877218271296521</v>
       </c>
       <c r="GE69" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="GF69" t="n">
         <v>-2.735722718354725e-05</v>
@@ -36626,13 +36698,13 @@
         <v>0</v>
       </c>
       <c r="GM69" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="GN69" t="n">
         <v>-0.02188938483799282</v>
       </c>
       <c r="GO69" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="GP69" t="n">
         <v>-7.302568026417882e-06</v>
@@ -36656,13 +36728,13 @@
         <v>0</v>
       </c>
       <c r="GW69" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="GX69" t="n">
         <v>-0.05949964923978149</v>
       </c>
       <c r="GY69" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="GZ69" t="n">
         <v>-0.008789671037433821</v>
@@ -36686,13 +36758,13 @@
         <v>0</v>
       </c>
       <c r="HG69" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="HH69" t="n">
         <v>-0.02395521864642743</v>
       </c>
       <c r="HI69" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="HJ69" t="n">
         <v>-6.799683141396897e-05</v>
@@ -36701,7 +36773,7 @@
         <v>0</v>
       </c>
       <c r="HL69" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="HM69" t="n">
         <v>0.06622564460675992</v>
@@ -36716,13 +36788,13 @@
         <v>0</v>
       </c>
       <c r="HQ69" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="HR69" t="n">
         <v>-0.03327358386716624</v>
       </c>
       <c r="HS69" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="HT69" t="n">
         <v>-0.0002485886090894331</v>
@@ -36821,7 +36893,7 @@
         <v>0</v>
       </c>
       <c r="IZ69" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="JA69" t="n">
         <v>0.09464502534016593</v>
@@ -36831,6 +36903,1783 @@
       </c>
       <c r="JC69" t="n">
         <v>6.101490173532565e-05</v>
+      </c>
+      <c r="JD69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2026-04-20 20:28:39</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>10</v>
+      </c>
+      <c r="C70" t="n">
+        <v>100</v>
+      </c>
+      <c r="D70" t="n">
+        <v>50</v>
+      </c>
+      <c r="E70" t="n">
+        <v>40</v>
+      </c>
+      <c r="F70" t="inlineStr"/>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>exp</t>
+        </is>
+      </c>
+      <c r="H70" t="n">
+        <v>0.1251436123068011</v>
+      </c>
+      <c r="I70" t="n">
+        <v>0.4166666666666667</v>
+      </c>
+      <c r="J70" t="n">
+        <v>0.9587027027027027</v>
+      </c>
+      <c r="K70" t="inlineStr"/>
+      <c r="L70" t="inlineStr"/>
+      <c r="M70" t="n">
+        <v>0.1643965840185594</v>
+      </c>
+      <c r="N70" t="n">
+        <v>0.4472135954999579</v>
+      </c>
+      <c r="O70" t="n">
+        <v>0.4227645714217698</v>
+      </c>
+      <c r="P70" t="inlineStr"/>
+      <c r="Q70" t="inlineStr"/>
+      <c r="R70" t="n">
+        <v>0.4536182413498976</v>
+      </c>
+      <c r="S70" t="n">
+        <v>0.4472135954999579</v>
+      </c>
+      <c r="T70" t="n">
+        <v>0.4476057660138444</v>
+      </c>
+      <c r="U70" t="inlineStr"/>
+      <c r="V70" t="inlineStr"/>
+      <c r="W70" t="n">
+        <v>0.4682029914119304</v>
+      </c>
+      <c r="X70" t="n">
+        <v>0.4472135954999579</v>
+      </c>
+      <c r="Y70" t="n">
+        <v>0.3903109310406991</v>
+      </c>
+      <c r="Z70" t="inlineStr"/>
+      <c r="AA70" t="inlineStr"/>
+      <c r="AB70" t="n">
+        <v>0.3013370522744404</v>
+      </c>
+      <c r="AC70" t="n">
+        <v>0.4472135954999579</v>
+      </c>
+      <c r="AD70" t="n">
+        <v>0.4628547114227459</v>
+      </c>
+      <c r="AE70" t="inlineStr"/>
+      <c r="AF70" t="inlineStr"/>
+      <c r="AG70" t="n">
+        <v>0.4651808420767356</v>
+      </c>
+      <c r="AH70" t="n">
+        <v>0.4472135954999579</v>
+      </c>
+      <c r="AI70" t="n">
+        <v>0.4950225526075757</v>
+      </c>
+      <c r="AJ70" t="inlineStr"/>
+      <c r="AK70" t="inlineStr"/>
+      <c r="AL70" t="n">
+        <v>0.5175120648629646</v>
+      </c>
+      <c r="AM70" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN70" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO70" t="inlineStr"/>
+      <c r="AP70" t="inlineStr"/>
+      <c r="AQ70" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR70" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS70" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT70" t="inlineStr"/>
+      <c r="AU70" t="inlineStr"/>
+      <c r="AV70" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW70" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX70" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY70" t="inlineStr"/>
+      <c r="AZ70" t="inlineStr"/>
+      <c r="BA70" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB70" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC70" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD70" t="inlineStr"/>
+      <c r="BE70" t="inlineStr"/>
+      <c r="BF70" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG70" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH70" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI70" t="inlineStr"/>
+      <c r="BJ70" t="inlineStr"/>
+      <c r="BK70" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL70" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM70" t="n">
+        <v>0.01142490100407152</v>
+      </c>
+      <c r="BN70" t="inlineStr"/>
+      <c r="BO70" t="inlineStr"/>
+      <c r="BP70" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ70" t="n">
+        <v>0</v>
+      </c>
+      <c r="BR70" t="n">
+        <v>0.04335391656419746</v>
+      </c>
+      <c r="BS70" t="inlineStr"/>
+      <c r="BT70" t="inlineStr"/>
+      <c r="BU70" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV70" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW70" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX70" t="inlineStr"/>
+      <c r="BY70" t="inlineStr"/>
+      <c r="BZ70" t="n">
+        <v>0</v>
+      </c>
+      <c r="CA70" t="n">
+        <v>0</v>
+      </c>
+      <c r="CB70" t="n">
+        <v>0</v>
+      </c>
+      <c r="CC70" t="inlineStr"/>
+      <c r="CD70" t="inlineStr"/>
+      <c r="CE70" t="n">
+        <v>0</v>
+      </c>
+      <c r="CF70" t="n">
+        <v>0</v>
+      </c>
+      <c r="CG70" t="n">
+        <v>0</v>
+      </c>
+      <c r="CH70" t="inlineStr"/>
+      <c r="CI70" t="inlineStr"/>
+      <c r="CJ70" t="n">
+        <v>0</v>
+      </c>
+      <c r="CK70" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL70" t="n">
+        <v>0.009399380166522486</v>
+      </c>
+      <c r="CM70" t="inlineStr"/>
+      <c r="CN70" t="inlineStr"/>
+      <c r="CO70" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP70" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ70" t="n">
+        <v>0.009784119489788528</v>
+      </c>
+      <c r="CR70" t="inlineStr"/>
+      <c r="CS70" t="inlineStr"/>
+      <c r="CT70" t="n">
+        <v>0</v>
+      </c>
+      <c r="CU70" t="n">
+        <v>0</v>
+      </c>
+      <c r="CV70" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW70" t="inlineStr"/>
+      <c r="CX70" t="inlineStr"/>
+      <c r="CY70" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ70" t="n">
+        <v>0</v>
+      </c>
+      <c r="DA70" t="n">
+        <v>0</v>
+      </c>
+      <c r="DB70" t="inlineStr"/>
+      <c r="DC70" t="inlineStr"/>
+      <c r="DD70" t="n">
+        <v>0</v>
+      </c>
+      <c r="DE70" t="n">
+        <v>0</v>
+      </c>
+      <c r="DF70" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG70" t="inlineStr"/>
+      <c r="DH70" t="inlineStr"/>
+      <c r="DI70" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ70" t="n">
+        <v>0</v>
+      </c>
+      <c r="DK70" t="n">
+        <v>0</v>
+      </c>
+      <c r="DL70" t="inlineStr"/>
+      <c r="DM70" t="inlineStr"/>
+      <c r="DN70" t="n">
+        <v>0</v>
+      </c>
+      <c r="DO70" t="n">
+        <v>0</v>
+      </c>
+      <c r="DP70" t="n">
+        <v>0</v>
+      </c>
+      <c r="DQ70" t="inlineStr"/>
+      <c r="DR70" t="inlineStr"/>
+      <c r="DS70" t="n">
+        <v>0</v>
+      </c>
+      <c r="DT70" t="n">
+        <v>0</v>
+      </c>
+      <c r="DU70" t="n">
+        <v>0</v>
+      </c>
+      <c r="DV70" t="inlineStr"/>
+      <c r="DW70" t="inlineStr"/>
+      <c r="DX70" t="n">
+        <v>0</v>
+      </c>
+      <c r="DY70" t="n">
+        <v>0</v>
+      </c>
+      <c r="DZ70" t="n">
+        <v>0.0145829241280647</v>
+      </c>
+      <c r="EA70" t="inlineStr"/>
+      <c r="EB70" t="inlineStr"/>
+      <c r="EC70" t="n">
+        <v>0</v>
+      </c>
+      <c r="ED70" t="n">
+        <v>0</v>
+      </c>
+      <c r="EE70" t="n">
+        <v>0</v>
+      </c>
+      <c r="EF70" t="inlineStr"/>
+      <c r="EG70" t="inlineStr"/>
+      <c r="EH70" t="n">
+        <v>0</v>
+      </c>
+      <c r="EI70" t="n">
+        <v>0</v>
+      </c>
+      <c r="EJ70" t="n">
+        <v>0</v>
+      </c>
+      <c r="EK70" t="inlineStr"/>
+      <c r="EL70" t="inlineStr"/>
+      <c r="EM70" t="n">
+        <v>0</v>
+      </c>
+      <c r="EN70" t="n">
+        <v>0</v>
+      </c>
+      <c r="EO70" t="n">
+        <v>0</v>
+      </c>
+      <c r="EP70" t="inlineStr"/>
+      <c r="EQ70" t="inlineStr"/>
+      <c r="ER70" t="n">
+        <v>0</v>
+      </c>
+      <c r="ES70" t="n">
+        <v>0</v>
+      </c>
+      <c r="ET70" t="n">
+        <v>0</v>
+      </c>
+      <c r="EU70" t="inlineStr"/>
+      <c r="EV70" t="inlineStr"/>
+      <c r="EW70" t="n">
+        <v>0</v>
+      </c>
+      <c r="EX70" t="n">
+        <v>0</v>
+      </c>
+      <c r="EY70" t="n">
+        <v>0</v>
+      </c>
+      <c r="EZ70" t="inlineStr"/>
+      <c r="FA70" t="inlineStr"/>
+      <c r="FB70" t="n">
+        <v>0</v>
+      </c>
+      <c r="FC70" t="n">
+        <v>0</v>
+      </c>
+      <c r="FD70" t="n">
+        <v>0</v>
+      </c>
+      <c r="FE70" t="inlineStr"/>
+      <c r="FF70" t="inlineStr"/>
+      <c r="FG70" t="n">
+        <v>0</v>
+      </c>
+      <c r="FH70" t="n">
+        <v>0</v>
+      </c>
+      <c r="FI70" t="n">
+        <v>0.0152037483177902</v>
+      </c>
+      <c r="FJ70" t="inlineStr"/>
+      <c r="FK70" t="inlineStr"/>
+      <c r="FL70" t="n">
+        <v>0</v>
+      </c>
+      <c r="FM70" t="n">
+        <v>0</v>
+      </c>
+      <c r="FN70" t="n">
+        <v>0.01223262848496849</v>
+      </c>
+      <c r="FO70" t="inlineStr"/>
+      <c r="FP70" t="inlineStr"/>
+      <c r="FQ70" t="n">
+        <v>0</v>
+      </c>
+      <c r="FR70" t="n">
+        <v>0</v>
+      </c>
+      <c r="FS70" t="n">
+        <v>0.02996838538756586</v>
+      </c>
+      <c r="FT70" t="inlineStr"/>
+      <c r="FU70" t="inlineStr"/>
+      <c r="FV70" t="n">
+        <v>0</v>
+      </c>
+      <c r="FW70" t="n">
+        <v>0</v>
+      </c>
+      <c r="FX70" t="n">
+        <v>0</v>
+      </c>
+      <c r="FY70" t="inlineStr"/>
+      <c r="FZ70" t="inlineStr"/>
+      <c r="GA70" t="n">
+        <v>0</v>
+      </c>
+      <c r="GB70" t="n">
+        <v>0</v>
+      </c>
+      <c r="GC70" t="n">
+        <v>0</v>
+      </c>
+      <c r="GD70" t="inlineStr"/>
+      <c r="GE70" t="inlineStr"/>
+      <c r="GF70" t="n">
+        <v>0</v>
+      </c>
+      <c r="GG70" t="n">
+        <v>0</v>
+      </c>
+      <c r="GH70" t="n">
+        <v>0.05091715384987692</v>
+      </c>
+      <c r="GI70" t="inlineStr"/>
+      <c r="GJ70" t="inlineStr"/>
+      <c r="GK70" t="n">
+        <v>0</v>
+      </c>
+      <c r="GL70" t="n">
+        <v>0</v>
+      </c>
+      <c r="GM70" t="n">
+        <v>0</v>
+      </c>
+      <c r="GN70" t="inlineStr"/>
+      <c r="GO70" t="inlineStr"/>
+      <c r="GP70" t="n">
+        <v>0</v>
+      </c>
+      <c r="GQ70" t="n">
+        <v>0</v>
+      </c>
+      <c r="GR70" t="n">
+        <v>0.03854382673323793</v>
+      </c>
+      <c r="GS70" t="inlineStr"/>
+      <c r="GT70" t="inlineStr"/>
+      <c r="GU70" t="n">
+        <v>0</v>
+      </c>
+      <c r="GV70" t="n">
+        <v>0</v>
+      </c>
+      <c r="GW70" t="n">
+        <v>0</v>
+      </c>
+      <c r="GX70" t="inlineStr"/>
+      <c r="GY70" t="inlineStr"/>
+      <c r="GZ70" t="n">
+        <v>0</v>
+      </c>
+      <c r="HA70" t="n">
+        <v>0</v>
+      </c>
+      <c r="HB70" t="n">
+        <v>0.02629735766088426</v>
+      </c>
+      <c r="HC70" t="inlineStr"/>
+      <c r="HD70" t="inlineStr"/>
+      <c r="HE70" t="n">
+        <v>0</v>
+      </c>
+      <c r="HF70" t="n">
+        <v>0</v>
+      </c>
+      <c r="HG70" t="n">
+        <v>0.01676969468782597</v>
+      </c>
+      <c r="HH70" t="inlineStr"/>
+      <c r="HI70" t="inlineStr"/>
+      <c r="HJ70" t="n">
+        <v>0</v>
+      </c>
+      <c r="HK70" t="n">
+        <v>0</v>
+      </c>
+      <c r="HL70" t="n">
+        <v>0</v>
+      </c>
+      <c r="HM70" t="inlineStr"/>
+      <c r="HN70" t="inlineStr"/>
+      <c r="HO70" t="n">
+        <v>0</v>
+      </c>
+      <c r="HP70" t="n">
+        <v>0</v>
+      </c>
+      <c r="HQ70" t="n">
+        <v>0.01569740142883769</v>
+      </c>
+      <c r="HR70" t="inlineStr"/>
+      <c r="HS70" t="inlineStr"/>
+      <c r="HT70" t="n">
+        <v>0</v>
+      </c>
+      <c r="HU70" t="n">
+        <v>0</v>
+      </c>
+      <c r="HV70" t="n">
+        <v>0</v>
+      </c>
+      <c r="HW70" t="inlineStr"/>
+      <c r="HX70" t="inlineStr"/>
+      <c r="HY70" t="n">
+        <v>0</v>
+      </c>
+      <c r="HZ70" t="n">
+        <v>0</v>
+      </c>
+      <c r="IA70" t="n">
+        <v>0</v>
+      </c>
+      <c r="IB70" t="inlineStr"/>
+      <c r="IC70" t="inlineStr"/>
+      <c r="ID70" t="n">
+        <v>0</v>
+      </c>
+      <c r="IE70" t="n">
+        <v>0</v>
+      </c>
+      <c r="IF70" t="n">
+        <v>0</v>
+      </c>
+      <c r="IG70" t="inlineStr"/>
+      <c r="IH70" t="inlineStr"/>
+      <c r="II70" t="n">
+        <v>0</v>
+      </c>
+      <c r="IJ70" t="n">
+        <v>0</v>
+      </c>
+      <c r="IK70" t="n">
+        <v>0.01765420746107408</v>
+      </c>
+      <c r="IL70" t="inlineStr"/>
+      <c r="IM70" t="inlineStr"/>
+      <c r="IN70" t="n">
+        <v>0</v>
+      </c>
+      <c r="IO70" t="n">
+        <v>0</v>
+      </c>
+      <c r="IP70" t="n">
+        <v>0</v>
+      </c>
+      <c r="IQ70" t="inlineStr"/>
+      <c r="IR70" t="inlineStr"/>
+      <c r="IS70" t="n">
+        <v>0</v>
+      </c>
+      <c r="IT70" t="n">
+        <v>0</v>
+      </c>
+      <c r="IU70" t="n">
+        <v>0</v>
+      </c>
+      <c r="IV70" t="inlineStr"/>
+      <c r="IW70" t="inlineStr"/>
+      <c r="IX70" t="n">
+        <v>0</v>
+      </c>
+      <c r="IY70" t="n">
+        <v>0</v>
+      </c>
+      <c r="IZ70" t="n">
+        <v>0</v>
+      </c>
+      <c r="JA70" t="inlineStr"/>
+      <c r="JB70" t="inlineStr"/>
+      <c r="JC70" t="n">
+        <v>0</v>
+      </c>
+      <c r="JD70" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-04-20 20:30:41</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>10</v>
+      </c>
+      <c r="C71" t="n">
+        <v>100</v>
+      </c>
+      <c r="D71" t="n">
+        <v>50</v>
+      </c>
+      <c r="E71" t="n">
+        <v>40</v>
+      </c>
+      <c r="F71" t="inlineStr"/>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>t1</t>
+        </is>
+      </c>
+      <c r="H71" t="n">
+        <v>0.3370658791072577</v>
+      </c>
+      <c r="I71" t="n">
+        <v>1</v>
+      </c>
+      <c r="J71" t="n">
+        <v>0.9160920920920921</v>
+      </c>
+      <c r="K71" t="inlineStr"/>
+      <c r="L71" t="inlineStr"/>
+      <c r="M71" t="n">
+        <v>0.3357806908995257</v>
+      </c>
+      <c r="N71" t="n">
+        <v>0.4472135954999579</v>
+      </c>
+      <c r="O71" t="n">
+        <v>0.2116385658378677</v>
+      </c>
+      <c r="P71" t="inlineStr"/>
+      <c r="Q71" t="inlineStr"/>
+      <c r="R71" t="n">
+        <v>0.1401070282539275</v>
+      </c>
+      <c r="S71" t="n">
+        <v>0.4472135954999579</v>
+      </c>
+      <c r="T71" t="n">
+        <v>0.4483099162127231</v>
+      </c>
+      <c r="U71" t="inlineStr"/>
+      <c r="V71" t="inlineStr"/>
+      <c r="W71" t="n">
+        <v>0.5138408309950322</v>
+      </c>
+      <c r="X71" t="n">
+        <v>0.4472135954999579</v>
+      </c>
+      <c r="Y71" t="n">
+        <v>0.4582588207412475</v>
+      </c>
+      <c r="Z71" t="inlineStr"/>
+      <c r="AA71" t="inlineStr"/>
+      <c r="AB71" t="n">
+        <v>0.445665023598454</v>
+      </c>
+      <c r="AC71" t="n">
+        <v>0.4472135954999579</v>
+      </c>
+      <c r="AD71" t="n">
+        <v>0.3320980017148263</v>
+      </c>
+      <c r="AE71" t="inlineStr"/>
+      <c r="AF71" t="inlineStr"/>
+      <c r="AG71" t="n">
+        <v>0.444911147462784</v>
+      </c>
+      <c r="AH71" t="n">
+        <v>0.4472135954999579</v>
+      </c>
+      <c r="AI71" t="n">
+        <v>0.6587390225478212</v>
+      </c>
+      <c r="AJ71" t="inlineStr"/>
+      <c r="AK71" t="inlineStr"/>
+      <c r="AL71" t="n">
+        <v>0.5654816845337634</v>
+      </c>
+      <c r="AM71" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN71" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO71" t="inlineStr"/>
+      <c r="AP71" t="inlineStr"/>
+      <c r="AQ71" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR71" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS71" t="n">
+        <v>1.273591312310204e-05</v>
+      </c>
+      <c r="AT71" t="inlineStr"/>
+      <c r="AU71" t="inlineStr"/>
+      <c r="AV71" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW71" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX71" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY71" t="inlineStr"/>
+      <c r="AZ71" t="inlineStr"/>
+      <c r="BA71" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB71" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC71" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD71" t="inlineStr"/>
+      <c r="BE71" t="inlineStr"/>
+      <c r="BF71" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG71" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH71" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI71" t="inlineStr"/>
+      <c r="BJ71" t="inlineStr"/>
+      <c r="BK71" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL71" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM71" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN71" t="inlineStr"/>
+      <c r="BO71" t="inlineStr"/>
+      <c r="BP71" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ71" t="n">
+        <v>0</v>
+      </c>
+      <c r="BR71" t="n">
+        <v>0</v>
+      </c>
+      <c r="BS71" t="inlineStr"/>
+      <c r="BT71" t="inlineStr"/>
+      <c r="BU71" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV71" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW71" t="n">
+        <v>8.335421681426141e-05</v>
+      </c>
+      <c r="BX71" t="inlineStr"/>
+      <c r="BY71" t="inlineStr"/>
+      <c r="BZ71" t="n">
+        <v>0</v>
+      </c>
+      <c r="CA71" t="n">
+        <v>0</v>
+      </c>
+      <c r="CB71" t="n">
+        <v>0</v>
+      </c>
+      <c r="CC71" t="inlineStr"/>
+      <c r="CD71" t="inlineStr"/>
+      <c r="CE71" t="n">
+        <v>0</v>
+      </c>
+      <c r="CF71" t="n">
+        <v>0</v>
+      </c>
+      <c r="CG71" t="n">
+        <v>0</v>
+      </c>
+      <c r="CH71" t="inlineStr"/>
+      <c r="CI71" t="inlineStr"/>
+      <c r="CJ71" t="n">
+        <v>0</v>
+      </c>
+      <c r="CK71" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL71" t="n">
+        <v>0</v>
+      </c>
+      <c r="CM71" t="inlineStr"/>
+      <c r="CN71" t="inlineStr"/>
+      <c r="CO71" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP71" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ71" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR71" t="inlineStr"/>
+      <c r="CS71" t="inlineStr"/>
+      <c r="CT71" t="n">
+        <v>0</v>
+      </c>
+      <c r="CU71" t="n">
+        <v>0</v>
+      </c>
+      <c r="CV71" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW71" t="inlineStr"/>
+      <c r="CX71" t="inlineStr"/>
+      <c r="CY71" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ71" t="n">
+        <v>0</v>
+      </c>
+      <c r="DA71" t="n">
+        <v>0</v>
+      </c>
+      <c r="DB71" t="inlineStr"/>
+      <c r="DC71" t="inlineStr"/>
+      <c r="DD71" t="n">
+        <v>0</v>
+      </c>
+      <c r="DE71" t="n">
+        <v>0</v>
+      </c>
+      <c r="DF71" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG71" t="inlineStr"/>
+      <c r="DH71" t="inlineStr"/>
+      <c r="DI71" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ71" t="n">
+        <v>0</v>
+      </c>
+      <c r="DK71" t="n">
+        <v>0</v>
+      </c>
+      <c r="DL71" t="inlineStr"/>
+      <c r="DM71" t="inlineStr"/>
+      <c r="DN71" t="n">
+        <v>0</v>
+      </c>
+      <c r="DO71" t="n">
+        <v>0</v>
+      </c>
+      <c r="DP71" t="n">
+        <v>0</v>
+      </c>
+      <c r="DQ71" t="inlineStr"/>
+      <c r="DR71" t="inlineStr"/>
+      <c r="DS71" t="n">
+        <v>0</v>
+      </c>
+      <c r="DT71" t="n">
+        <v>0</v>
+      </c>
+      <c r="DU71" t="n">
+        <v>0</v>
+      </c>
+      <c r="DV71" t="inlineStr"/>
+      <c r="DW71" t="inlineStr"/>
+      <c r="DX71" t="n">
+        <v>0</v>
+      </c>
+      <c r="DY71" t="n">
+        <v>0</v>
+      </c>
+      <c r="DZ71" t="n">
+        <v>0</v>
+      </c>
+      <c r="EA71" t="inlineStr"/>
+      <c r="EB71" t="inlineStr"/>
+      <c r="EC71" t="n">
+        <v>0</v>
+      </c>
+      <c r="ED71" t="n">
+        <v>0</v>
+      </c>
+      <c r="EE71" t="n">
+        <v>0</v>
+      </c>
+      <c r="EF71" t="inlineStr"/>
+      <c r="EG71" t="inlineStr"/>
+      <c r="EH71" t="n">
+        <v>0</v>
+      </c>
+      <c r="EI71" t="n">
+        <v>0</v>
+      </c>
+      <c r="EJ71" t="n">
+        <v>0</v>
+      </c>
+      <c r="EK71" t="inlineStr"/>
+      <c r="EL71" t="inlineStr"/>
+      <c r="EM71" t="n">
+        <v>0</v>
+      </c>
+      <c r="EN71" t="n">
+        <v>0</v>
+      </c>
+      <c r="EO71" t="n">
+        <v>0</v>
+      </c>
+      <c r="EP71" t="inlineStr"/>
+      <c r="EQ71" t="inlineStr"/>
+      <c r="ER71" t="n">
+        <v>0</v>
+      </c>
+      <c r="ES71" t="n">
+        <v>0</v>
+      </c>
+      <c r="ET71" t="n">
+        <v>0</v>
+      </c>
+      <c r="EU71" t="inlineStr"/>
+      <c r="EV71" t="inlineStr"/>
+      <c r="EW71" t="n">
+        <v>0</v>
+      </c>
+      <c r="EX71" t="n">
+        <v>0</v>
+      </c>
+      <c r="EY71" t="n">
+        <v>0</v>
+      </c>
+      <c r="EZ71" t="inlineStr"/>
+      <c r="FA71" t="inlineStr"/>
+      <c r="FB71" t="n">
+        <v>0</v>
+      </c>
+      <c r="FC71" t="n">
+        <v>0</v>
+      </c>
+      <c r="FD71" t="n">
+        <v>0</v>
+      </c>
+      <c r="FE71" t="inlineStr"/>
+      <c r="FF71" t="inlineStr"/>
+      <c r="FG71" t="n">
+        <v>0</v>
+      </c>
+      <c r="FH71" t="n">
+        <v>0</v>
+      </c>
+      <c r="FI71" t="n">
+        <v>0</v>
+      </c>
+      <c r="FJ71" t="inlineStr"/>
+      <c r="FK71" t="inlineStr"/>
+      <c r="FL71" t="n">
+        <v>0</v>
+      </c>
+      <c r="FM71" t="n">
+        <v>0</v>
+      </c>
+      <c r="FN71" t="n">
+        <v>0</v>
+      </c>
+      <c r="FO71" t="inlineStr"/>
+      <c r="FP71" t="inlineStr"/>
+      <c r="FQ71" t="n">
+        <v>0</v>
+      </c>
+      <c r="FR71" t="n">
+        <v>0</v>
+      </c>
+      <c r="FS71" t="n">
+        <v>0</v>
+      </c>
+      <c r="FT71" t="inlineStr"/>
+      <c r="FU71" t="inlineStr"/>
+      <c r="FV71" t="n">
+        <v>0</v>
+      </c>
+      <c r="FW71" t="n">
+        <v>0</v>
+      </c>
+      <c r="FX71" t="n">
+        <v>0</v>
+      </c>
+      <c r="FY71" t="inlineStr"/>
+      <c r="FZ71" t="inlineStr"/>
+      <c r="GA71" t="n">
+        <v>0</v>
+      </c>
+      <c r="GB71" t="n">
+        <v>0</v>
+      </c>
+      <c r="GC71" t="n">
+        <v>2.475974687393181e-06</v>
+      </c>
+      <c r="GD71" t="inlineStr"/>
+      <c r="GE71" t="inlineStr"/>
+      <c r="GF71" t="n">
+        <v>0</v>
+      </c>
+      <c r="GG71" t="n">
+        <v>0</v>
+      </c>
+      <c r="GH71" t="n">
+        <v>0</v>
+      </c>
+      <c r="GI71" t="inlineStr"/>
+      <c r="GJ71" t="inlineStr"/>
+      <c r="GK71" t="n">
+        <v>0</v>
+      </c>
+      <c r="GL71" t="n">
+        <v>0</v>
+      </c>
+      <c r="GM71" t="n">
+        <v>0</v>
+      </c>
+      <c r="GN71" t="inlineStr"/>
+      <c r="GO71" t="inlineStr"/>
+      <c r="GP71" t="n">
+        <v>0</v>
+      </c>
+      <c r="GQ71" t="n">
+        <v>0</v>
+      </c>
+      <c r="GR71" t="n">
+        <v>0</v>
+      </c>
+      <c r="GS71" t="inlineStr"/>
+      <c r="GT71" t="inlineStr"/>
+      <c r="GU71" t="n">
+        <v>0</v>
+      </c>
+      <c r="GV71" t="n">
+        <v>0</v>
+      </c>
+      <c r="GW71" t="n">
+        <v>0</v>
+      </c>
+      <c r="GX71" t="inlineStr"/>
+      <c r="GY71" t="inlineStr"/>
+      <c r="GZ71" t="n">
+        <v>0</v>
+      </c>
+      <c r="HA71" t="n">
+        <v>0</v>
+      </c>
+      <c r="HB71" t="n">
+        <v>0</v>
+      </c>
+      <c r="HC71" t="inlineStr"/>
+      <c r="HD71" t="inlineStr"/>
+      <c r="HE71" t="n">
+        <v>0</v>
+      </c>
+      <c r="HF71" t="n">
+        <v>0</v>
+      </c>
+      <c r="HG71" t="n">
+        <v>0</v>
+      </c>
+      <c r="HH71" t="inlineStr"/>
+      <c r="HI71" t="inlineStr"/>
+      <c r="HJ71" t="n">
+        <v>0</v>
+      </c>
+      <c r="HK71" t="n">
+        <v>0</v>
+      </c>
+      <c r="HL71" t="n">
+        <v>0</v>
+      </c>
+      <c r="HM71" t="inlineStr"/>
+      <c r="HN71" t="inlineStr"/>
+      <c r="HO71" t="n">
+        <v>0</v>
+      </c>
+      <c r="HP71" t="n">
+        <v>0</v>
+      </c>
+      <c r="HQ71" t="n">
+        <v>0</v>
+      </c>
+      <c r="HR71" t="inlineStr"/>
+      <c r="HS71" t="inlineStr"/>
+      <c r="HT71" t="n">
+        <v>0</v>
+      </c>
+      <c r="HU71" t="n">
+        <v>0</v>
+      </c>
+      <c r="HV71" t="n">
+        <v>0</v>
+      </c>
+      <c r="HW71" t="inlineStr"/>
+      <c r="HX71" t="inlineStr"/>
+      <c r="HY71" t="n">
+        <v>0</v>
+      </c>
+      <c r="HZ71" t="n">
+        <v>0</v>
+      </c>
+      <c r="IA71" t="n">
+        <v>0</v>
+      </c>
+      <c r="IB71" t="inlineStr"/>
+      <c r="IC71" t="inlineStr"/>
+      <c r="ID71" t="n">
+        <v>0</v>
+      </c>
+      <c r="IE71" t="n">
+        <v>0</v>
+      </c>
+      <c r="IF71" t="n">
+        <v>0</v>
+      </c>
+      <c r="IG71" t="inlineStr"/>
+      <c r="IH71" t="inlineStr"/>
+      <c r="II71" t="n">
+        <v>0</v>
+      </c>
+      <c r="IJ71" t="n">
+        <v>0</v>
+      </c>
+      <c r="IK71" t="n">
+        <v>0</v>
+      </c>
+      <c r="IL71" t="inlineStr"/>
+      <c r="IM71" t="inlineStr"/>
+      <c r="IN71" t="n">
+        <v>0</v>
+      </c>
+      <c r="IO71" t="n">
+        <v>0</v>
+      </c>
+      <c r="IP71" t="n">
+        <v>1.331896293025564e-06</v>
+      </c>
+      <c r="IQ71" t="inlineStr"/>
+      <c r="IR71" t="inlineStr"/>
+      <c r="IS71" t="n">
+        <v>0</v>
+      </c>
+      <c r="IT71" t="n">
+        <v>0</v>
+      </c>
+      <c r="IU71" t="n">
+        <v>0</v>
+      </c>
+      <c r="IV71" t="inlineStr"/>
+      <c r="IW71" t="inlineStr"/>
+      <c r="IX71" t="n">
+        <v>0</v>
+      </c>
+      <c r="IY71" t="n">
+        <v>0</v>
+      </c>
+      <c r="IZ71" t="n">
+        <v>0</v>
+      </c>
+      <c r="JA71" t="inlineStr"/>
+      <c r="JB71" t="inlineStr"/>
+      <c r="JC71" t="n">
+        <v>0</v>
+      </c>
+      <c r="JD71" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2026-04-20 20:32:38</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>10</v>
+      </c>
+      <c r="C72" t="n">
+        <v>100</v>
+      </c>
+      <c r="D72" t="n">
+        <v>50</v>
+      </c>
+      <c r="E72" t="n">
+        <v>40</v>
+      </c>
+      <c r="F72" t="inlineStr"/>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>t1</t>
+        </is>
+      </c>
+      <c r="H72" t="n">
+        <v>0.2212412936712705</v>
+      </c>
+      <c r="I72" t="n">
+        <v>0.7692307692307693</v>
+      </c>
+      <c r="J72" t="n">
+        <v>0.9484164164164164</v>
+      </c>
+      <c r="K72" t="inlineStr"/>
+      <c r="L72" t="inlineStr"/>
+      <c r="M72" t="n">
+        <v>0.2094488497938567</v>
+      </c>
+      <c r="N72" t="n">
+        <v>0.4472135954999579</v>
+      </c>
+      <c r="O72" t="n">
+        <v>0.345213720537687</v>
+      </c>
+      <c r="P72" t="inlineStr"/>
+      <c r="Q72" t="inlineStr"/>
+      <c r="R72" t="n">
+        <v>0.2621197160845905</v>
+      </c>
+      <c r="S72" t="n">
+        <v>0.4472135954999579</v>
+      </c>
+      <c r="T72" t="n">
+        <v>0.4497934977411436</v>
+      </c>
+      <c r="U72" t="inlineStr"/>
+      <c r="V72" t="inlineStr"/>
+      <c r="W72" t="n">
+        <v>0.4933906744900063</v>
+      </c>
+      <c r="X72" t="n">
+        <v>0.4472135954999579</v>
+      </c>
+      <c r="Y72" t="n">
+        <v>0.4481342723497151</v>
+      </c>
+      <c r="Z72" t="inlineStr"/>
+      <c r="AA72" t="inlineStr"/>
+      <c r="AB72" t="n">
+        <v>0.4510745601421027</v>
+      </c>
+      <c r="AC72" t="n">
+        <v>0.4472135954999579</v>
+      </c>
+      <c r="AD72" t="n">
+        <v>0.3912981498055055</v>
+      </c>
+      <c r="AE72" t="inlineStr"/>
+      <c r="AF72" t="inlineStr"/>
+      <c r="AG72" t="n">
+        <v>0.4468367471272708</v>
+      </c>
+      <c r="AH72" t="n">
+        <v>0.4472135954999579</v>
+      </c>
+      <c r="AI72" t="n">
+        <v>0.5469031335859372</v>
+      </c>
+      <c r="AJ72" t="inlineStr"/>
+      <c r="AK72" t="inlineStr"/>
+      <c r="AL72" t="n">
+        <v>0.5335947554610392</v>
+      </c>
+      <c r="AM72" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN72" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO72" t="inlineStr"/>
+      <c r="AP72" t="inlineStr"/>
+      <c r="AQ72" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR72" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS72" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT72" t="inlineStr"/>
+      <c r="AU72" t="inlineStr"/>
+      <c r="AV72" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW72" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX72" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY72" t="inlineStr"/>
+      <c r="AZ72" t="inlineStr"/>
+      <c r="BA72" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB72" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC72" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD72" t="inlineStr"/>
+      <c r="BE72" t="inlineStr"/>
+      <c r="BF72" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG72" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH72" t="n">
+        <v>-0</v>
+      </c>
+      <c r="BI72" t="inlineStr"/>
+      <c r="BJ72" t="inlineStr"/>
+      <c r="BK72" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL72" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM72" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN72" t="inlineStr"/>
+      <c r="BO72" t="inlineStr"/>
+      <c r="BP72" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ72" t="n">
+        <v>0</v>
+      </c>
+      <c r="BR72" t="n">
+        <v>0</v>
+      </c>
+      <c r="BS72" t="inlineStr"/>
+      <c r="BT72" t="inlineStr"/>
+      <c r="BU72" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV72" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW72" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX72" t="inlineStr"/>
+      <c r="BY72" t="inlineStr"/>
+      <c r="BZ72" t="n">
+        <v>0</v>
+      </c>
+      <c r="CA72" t="n">
+        <v>0</v>
+      </c>
+      <c r="CB72" t="n">
+        <v>-0</v>
+      </c>
+      <c r="CC72" t="inlineStr"/>
+      <c r="CD72" t="inlineStr"/>
+      <c r="CE72" t="n">
+        <v>0</v>
+      </c>
+      <c r="CF72" t="n">
+        <v>0</v>
+      </c>
+      <c r="CG72" t="n">
+        <v>0</v>
+      </c>
+      <c r="CH72" t="inlineStr"/>
+      <c r="CI72" t="inlineStr"/>
+      <c r="CJ72" t="n">
+        <v>0</v>
+      </c>
+      <c r="CK72" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL72" t="n">
+        <v>-0.03265120641357604</v>
+      </c>
+      <c r="CM72" t="inlineStr"/>
+      <c r="CN72" t="inlineStr"/>
+      <c r="CO72" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP72" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ72" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR72" t="inlineStr"/>
+      <c r="CS72" t="inlineStr"/>
+      <c r="CT72" t="n">
+        <v>0</v>
+      </c>
+      <c r="CU72" t="n">
+        <v>0</v>
+      </c>
+      <c r="CV72" t="n">
+        <v>-0</v>
+      </c>
+      <c r="CW72" t="inlineStr"/>
+      <c r="CX72" t="inlineStr"/>
+      <c r="CY72" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ72" t="n">
+        <v>0</v>
+      </c>
+      <c r="DA72" t="n">
+        <v>0</v>
+      </c>
+      <c r="DB72" t="inlineStr"/>
+      <c r="DC72" t="inlineStr"/>
+      <c r="DD72" t="n">
+        <v>0</v>
+      </c>
+      <c r="DE72" t="n">
+        <v>0</v>
+      </c>
+      <c r="DF72" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG72" t="inlineStr"/>
+      <c r="DH72" t="inlineStr"/>
+      <c r="DI72" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ72" t="n">
+        <v>0</v>
+      </c>
+      <c r="DK72" t="n">
+        <v>-0</v>
+      </c>
+      <c r="DL72" t="inlineStr"/>
+      <c r="DM72" t="inlineStr"/>
+      <c r="DN72" t="n">
+        <v>0</v>
+      </c>
+      <c r="DO72" t="n">
+        <v>0</v>
+      </c>
+      <c r="DP72" t="n">
+        <v>-0</v>
+      </c>
+      <c r="DQ72" t="inlineStr"/>
+      <c r="DR72" t="inlineStr"/>
+      <c r="DS72" t="n">
+        <v>0</v>
+      </c>
+      <c r="DT72" t="n">
+        <v>0</v>
+      </c>
+      <c r="DU72" t="n">
+        <v>0</v>
+      </c>
+      <c r="DV72" t="inlineStr"/>
+      <c r="DW72" t="inlineStr"/>
+      <c r="DX72" t="n">
+        <v>0</v>
+      </c>
+      <c r="DY72" t="n">
+        <v>0</v>
+      </c>
+      <c r="DZ72" t="n">
+        <v>0</v>
+      </c>
+      <c r="EA72" t="inlineStr"/>
+      <c r="EB72" t="inlineStr"/>
+      <c r="EC72" t="n">
+        <v>0</v>
+      </c>
+      <c r="ED72" t="n">
+        <v>0</v>
+      </c>
+      <c r="EE72" t="n">
+        <v>0</v>
+      </c>
+      <c r="EF72" t="inlineStr"/>
+      <c r="EG72" t="inlineStr"/>
+      <c r="EH72" t="n">
+        <v>0</v>
+      </c>
+      <c r="EI72" t="n">
+        <v>0</v>
+      </c>
+      <c r="EJ72" t="n">
+        <v>0</v>
+      </c>
+      <c r="EK72" t="inlineStr"/>
+      <c r="EL72" t="inlineStr"/>
+      <c r="EM72" t="n">
+        <v>0</v>
+      </c>
+      <c r="EN72" t="n">
+        <v>0</v>
+      </c>
+      <c r="EO72" t="n">
+        <v>0</v>
+      </c>
+      <c r="EP72" t="inlineStr"/>
+      <c r="EQ72" t="inlineStr"/>
+      <c r="ER72" t="n">
+        <v>0</v>
+      </c>
+      <c r="ES72" t="n">
+        <v>0</v>
+      </c>
+      <c r="ET72" t="n">
+        <v>-0.09037031430505783</v>
+      </c>
+      <c r="EU72" t="inlineStr"/>
+      <c r="EV72" t="inlineStr"/>
+      <c r="EW72" t="n">
+        <v>0</v>
+      </c>
+      <c r="EX72" t="n">
+        <v>0</v>
+      </c>
+      <c r="EY72" t="n">
+        <v>-0</v>
+      </c>
+      <c r="EZ72" t="inlineStr"/>
+      <c r="FA72" t="inlineStr"/>
+      <c r="FB72" t="n">
+        <v>0</v>
+      </c>
+      <c r="FC72" t="n">
+        <v>0</v>
+      </c>
+      <c r="FD72" t="n">
+        <v>0</v>
+      </c>
+      <c r="FE72" t="inlineStr"/>
+      <c r="FF72" t="inlineStr"/>
+      <c r="FG72" t="n">
+        <v>0</v>
+      </c>
+      <c r="FH72" t="n">
+        <v>0</v>
+      </c>
+      <c r="FI72" t="n">
+        <v>0</v>
+      </c>
+      <c r="FJ72" t="inlineStr"/>
+      <c r="FK72" t="inlineStr"/>
+      <c r="FL72" t="n">
+        <v>0</v>
+      </c>
+      <c r="FM72" t="n">
+        <v>0</v>
+      </c>
+      <c r="FN72" t="n">
+        <v>-0</v>
+      </c>
+      <c r="FO72" t="inlineStr"/>
+      <c r="FP72" t="inlineStr"/>
+      <c r="FQ72" t="n">
+        <v>0</v>
+      </c>
+      <c r="FR72" t="n">
+        <v>0</v>
+      </c>
+      <c r="FS72" t="n">
+        <v>-0</v>
+      </c>
+      <c r="FT72" t="inlineStr"/>
+      <c r="FU72" t="inlineStr"/>
+      <c r="FV72" t="n">
+        <v>0</v>
+      </c>
+      <c r="FW72" t="n">
+        <v>0</v>
+      </c>
+      <c r="FX72" t="n">
+        <v>-0</v>
+      </c>
+      <c r="FY72" t="inlineStr"/>
+      <c r="FZ72" t="inlineStr"/>
+      <c r="GA72" t="n">
+        <v>0</v>
+      </c>
+      <c r="GB72" t="n">
+        <v>0</v>
+      </c>
+      <c r="GC72" t="n">
+        <v>0</v>
+      </c>
+      <c r="GD72" t="inlineStr"/>
+      <c r="GE72" t="inlineStr"/>
+      <c r="GF72" t="n">
+        <v>0</v>
+      </c>
+      <c r="GG72" t="n">
+        <v>0</v>
+      </c>
+      <c r="GH72" t="n">
+        <v>0</v>
+      </c>
+      <c r="GI72" t="inlineStr"/>
+      <c r="GJ72" t="inlineStr"/>
+      <c r="GK72" t="n">
+        <v>0</v>
+      </c>
+      <c r="GL72" t="n">
+        <v>0</v>
+      </c>
+      <c r="GM72" t="n">
+        <v>0.1274315342470725</v>
+      </c>
+      <c r="GN72" t="inlineStr"/>
+      <c r="GO72" t="inlineStr"/>
+      <c r="GP72" t="n">
+        <v>0</v>
+      </c>
+      <c r="GQ72" t="n">
+        <v>0</v>
+      </c>
+      <c r="GR72" t="n">
+        <v>-0</v>
+      </c>
+      <c r="GS72" t="inlineStr"/>
+      <c r="GT72" t="inlineStr"/>
+      <c r="GU72" t="n">
+        <v>0</v>
+      </c>
+      <c r="GV72" t="n">
+        <v>0</v>
+      </c>
+      <c r="GW72" t="n">
+        <v>-0</v>
+      </c>
+      <c r="GX72" t="inlineStr"/>
+      <c r="GY72" t="inlineStr"/>
+      <c r="GZ72" t="n">
+        <v>0</v>
+      </c>
+      <c r="HA72" t="n">
+        <v>0</v>
+      </c>
+      <c r="HB72" t="n">
+        <v>0</v>
+      </c>
+      <c r="HC72" t="inlineStr"/>
+      <c r="HD72" t="inlineStr"/>
+      <c r="HE72" t="n">
+        <v>0</v>
+      </c>
+      <c r="HF72" t="n">
+        <v>0</v>
+      </c>
+      <c r="HG72" t="n">
+        <v>-0</v>
+      </c>
+      <c r="HH72" t="inlineStr"/>
+      <c r="HI72" t="inlineStr"/>
+      <c r="HJ72" t="n">
+        <v>0</v>
+      </c>
+      <c r="HK72" t="n">
+        <v>0</v>
+      </c>
+      <c r="HL72" t="n">
+        <v>0</v>
+      </c>
+      <c r="HM72" t="inlineStr"/>
+      <c r="HN72" t="inlineStr"/>
+      <c r="HO72" t="n">
+        <v>0</v>
+      </c>
+      <c r="HP72" t="n">
+        <v>0</v>
+      </c>
+      <c r="HQ72" t="n">
+        <v>0</v>
+      </c>
+      <c r="HR72" t="inlineStr"/>
+      <c r="HS72" t="inlineStr"/>
+      <c r="HT72" t="n">
+        <v>0</v>
+      </c>
+      <c r="HU72" t="n">
+        <v>0</v>
+      </c>
+      <c r="HV72" t="n">
+        <v>-0</v>
+      </c>
+      <c r="HW72" t="inlineStr"/>
+      <c r="HX72" t="inlineStr"/>
+      <c r="HY72" t="n">
+        <v>0</v>
+      </c>
+      <c r="HZ72" t="n">
+        <v>0</v>
+      </c>
+      <c r="IA72" t="n">
+        <v>0</v>
+      </c>
+      <c r="IB72" t="inlineStr"/>
+      <c r="IC72" t="inlineStr"/>
+      <c r="ID72" t="n">
+        <v>0</v>
+      </c>
+      <c r="IE72" t="n">
+        <v>0</v>
+      </c>
+      <c r="IF72" t="n">
+        <v>0</v>
+      </c>
+      <c r="IG72" t="inlineStr"/>
+      <c r="IH72" t="inlineStr"/>
+      <c r="II72" t="n">
+        <v>0</v>
+      </c>
+      <c r="IJ72" t="n">
+        <v>0</v>
+      </c>
+      <c r="IK72" t="n">
+        <v>0</v>
+      </c>
+      <c r="IL72" t="inlineStr"/>
+      <c r="IM72" t="inlineStr"/>
+      <c r="IN72" t="n">
+        <v>0</v>
+      </c>
+      <c r="IO72" t="n">
+        <v>0</v>
+      </c>
+      <c r="IP72" t="n">
+        <v>-3.486811104169365e-06</v>
+      </c>
+      <c r="IQ72" t="inlineStr"/>
+      <c r="IR72" t="inlineStr"/>
+      <c r="IS72" t="n">
+        <v>0</v>
+      </c>
+      <c r="IT72" t="n">
+        <v>0</v>
+      </c>
+      <c r="IU72" t="n">
+        <v>-0</v>
+      </c>
+      <c r="IV72" t="inlineStr"/>
+      <c r="IW72" t="inlineStr"/>
+      <c r="IX72" t="n">
+        <v>0</v>
+      </c>
+      <c r="IY72" t="n">
+        <v>0</v>
+      </c>
+      <c r="IZ72" t="n">
+        <v>0</v>
+      </c>
+      <c r="JA72" t="inlineStr"/>
+      <c r="JB72" t="inlineStr"/>
+      <c r="JC72" t="n">
+        <v>0</v>
+      </c>
+      <c r="JD72" t="n">
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>